<commit_message>
[Lane 1] USA26046 pig counts: second cost view with unrated pigs at same-size Pin rate
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02-facilities/Cenovus/Lima-OH/USA26046-pig-counts.xlsx
+++ b/02-facilities/Cenovus/Lima-OH/USA26046-pig-counts.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -475,6 +475,8 @@
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -542,6 +544,16 @@
           <t>New pigs with no rate</t>
         </is>
       </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Cost - new pigs, unrated at Pin rate (USD)</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>New pigs still with no rate</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -578,6 +590,14 @@
         <f>'Crude'!D32</f>
         <v/>
       </c>
+      <c r="K5" s="4">
+        <f>'Crude'!N31</f>
+        <v/>
+      </c>
+      <c r="L5">
+        <f>'Crude'!N32</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -614,6 +634,14 @@
         <f>'HDS'!D13</f>
         <v/>
       </c>
+      <c r="K6" s="4">
+        <f>'HDS'!N12</f>
+        <v/>
+      </c>
+      <c r="L6">
+        <f>'HDS'!N13</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -650,6 +678,14 @@
         <f>'Coker'!D49</f>
         <v/>
       </c>
+      <c r="K7" s="4">
+        <f>'Coker'!N48</f>
+        <v/>
+      </c>
+      <c r="L7">
+        <f>'Coker'!N49</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -686,6 +722,14 @@
         <f>'Vac'!D40</f>
         <v/>
       </c>
+      <c r="K8" s="4">
+        <f>'Vac'!N39</f>
+        <v/>
+      </c>
+      <c r="L8">
+        <f>'Vac'!N40</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -729,18 +773,26 @@
         <f>SUM(J5:J8)</f>
         <v/>
       </c>
+      <c r="K9" s="6">
+        <f>SUM(K5:K8)</f>
+        <v/>
+      </c>
+      <c r="L9" s="5">
+        <f>SUM(L5:L8)</f>
+        <v/>
+      </c>
     </row>
     <row r="11" ht="60" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Costing: New pigs only, at the pigs.xlsx rate for the same size and type; used pigs are not costed (Jesse, 2026-10-02). Bolted and HR pigs without their own rate take the same-size Pin rate (pigs.xlsx prices Bolt and HR the same as Pin wherever it lists both); Foam takes the Gauge Foam rate. Sizes or types not on pigs.xlsx carry no rate and are counted in "New pigs with no rate".</t>
+          <t>Costing: New pigs only, at the pigs.xlsx rate for the same size and type; used pigs are not costed (Jesse, 2026-10-02). Bolted and HR pigs without their own rate take the same-size Pin rate (pigs.xlsx prices Bolt and HR the same as Pin wherever it lists both); Foam takes the Gauge Foam rate. Sizes or types not on pigs.xlsx carry no rate and are counted in "New pigs with no rate". Second view (Jesse, 2026-10-02: admin may count them as Pin): rated pigs unchanged; unrated Pin/HR/FMJ/unclear pigs take the same-size Pin rate where pigs.xlsx has one. Foams, swabs and honeycomb are not repriced. Neither view is treated as the correct one.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A11:L11"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A11:J11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -752,7 +804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:N32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -767,6 +819,8 @@
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="30" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -837,6 +891,16 @@
           <t>Cost - new pigs (USD)</t>
         </is>
       </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>Rate - unrated pigs at Pin (USD)</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>Cost - new pigs, unrated at Pin rate (USD)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -880,6 +944,11 @@
         <f>IF(J3="","",D3*J3)</f>
         <v/>
       </c>
+      <c r="M3" s="4" t="n"/>
+      <c r="N3" s="4">
+        <f>IF(M3="","",D3*M3)</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
@@ -923,6 +992,11 @@
         <f>IF(J4="","",D4*J4)</f>
         <v/>
       </c>
+      <c r="M4" s="9" t="n"/>
+      <c r="N4" s="9">
+        <f>IF(M4="","",D4*M4)</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -968,6 +1042,13 @@
         <f>IF(J5="","",D5*J5)</f>
         <v/>
       </c>
+      <c r="M5" s="4" t="n">
+        <v>118</v>
+      </c>
+      <c r="N5" s="4">
+        <f>IF(M5="","",D5*M5)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
@@ -1013,6 +1094,13 @@
         <f>IF(J6="","",D6*J6)</f>
         <v/>
       </c>
+      <c r="M6" s="9" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="N6" s="9">
+        <f>IF(M6="","",D6*M6)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1058,6 +1146,13 @@
         <f>IF(J7="","",D7*J7)</f>
         <v/>
       </c>
+      <c r="M7" s="4" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="N7" s="4">
+        <f>IF(M7="","",D7*M7)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
@@ -1101,6 +1196,13 @@
         <f>IF(J8="","",D8*J8)</f>
         <v/>
       </c>
+      <c r="M8" s="9" t="n">
+        <v>118</v>
+      </c>
+      <c r="N8" s="9">
+        <f>IF(M8="","",D8*M8)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1146,6 +1248,13 @@
         <f>IF(J9="","",D9*J9)</f>
         <v/>
       </c>
+      <c r="M9" s="4" t="n">
+        <v>118</v>
+      </c>
+      <c r="N9" s="4">
+        <f>IF(M9="","",D9*M9)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
@@ -1191,6 +1300,13 @@
         <f>IF(J10="","",D10*J10)</f>
         <v/>
       </c>
+      <c r="M10" s="9" t="n">
+        <v>129.8</v>
+      </c>
+      <c r="N10" s="9">
+        <f>IF(M10="","",D10*M10)</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1236,6 +1352,13 @@
         <f>IF(J11="","",D11*J11)</f>
         <v/>
       </c>
+      <c r="M11" s="4" t="n">
+        <v>129.8</v>
+      </c>
+      <c r="N11" s="4">
+        <f>IF(M11="","",D11*M11)</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
@@ -1279,6 +1402,13 @@
         <f>IF(J12="","",D12*J12)</f>
         <v/>
       </c>
+      <c r="M12" s="9" t="n">
+        <v>129.8</v>
+      </c>
+      <c r="N12" s="9">
+        <f>IF(M12="","",D12*M12)</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1322,6 +1452,13 @@
         <f>IF(J13="","",D13*J13)</f>
         <v/>
       </c>
+      <c r="M13" s="4" t="n">
+        <v>129.8</v>
+      </c>
+      <c r="N13" s="4">
+        <f>IF(M13="","",D13*M13)</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
@@ -1367,6 +1504,13 @@
         <f>IF(J14="","",D14*J14)</f>
         <v/>
       </c>
+      <c r="M14" s="9" t="n">
+        <v>129.8</v>
+      </c>
+      <c r="N14" s="9">
+        <f>IF(M14="","",D14*M14)</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1410,6 +1554,11 @@
         <f>IF(J15="","",D15*J15)</f>
         <v/>
       </c>
+      <c r="M15" s="4" t="n"/>
+      <c r="N15" s="4">
+        <f>IF(M15="","",D15*M15)</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
@@ -1453,6 +1602,11 @@
         <f>IF(J16="","",D16*J16)</f>
         <v/>
       </c>
+      <c r="M16" s="9" t="n"/>
+      <c r="N16" s="9">
+        <f>IF(M16="","",D16*M16)</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1496,6 +1650,11 @@
         <f>IF(J17="","",D17*J17)</f>
         <v/>
       </c>
+      <c r="M17" s="4" t="n"/>
+      <c r="N17" s="4">
+        <f>IF(M17="","",D17*M17)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
@@ -1539,6 +1698,11 @@
         <f>IF(J18="","",D18*J18)</f>
         <v/>
       </c>
+      <c r="M18" s="9" t="n"/>
+      <c r="N18" s="9">
+        <f>IF(M18="","",D18*M18)</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1584,6 +1748,13 @@
         <f>IF(J19="","",D19*J19)</f>
         <v/>
       </c>
+      <c r="M19" s="4" t="n">
+        <v>230.1</v>
+      </c>
+      <c r="N19" s="4">
+        <f>IF(M19="","",D19*M19)</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
@@ -1627,6 +1798,13 @@
         <f>IF(J20="","",D20*J20)</f>
         <v/>
       </c>
+      <c r="M20" s="9" t="n">
+        <v>230.1</v>
+      </c>
+      <c r="N20" s="9">
+        <f>IF(M20="","",D20*M20)</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1670,6 +1848,13 @@
         <f>IF(J21="","",D21*J21)</f>
         <v/>
       </c>
+      <c r="M21" s="4" t="n">
+        <v>230.1</v>
+      </c>
+      <c r="N21" s="4">
+        <f>IF(M21="","",D21*M21)</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
@@ -1715,6 +1900,13 @@
         <f>IF(J22="","",D22*J22)</f>
         <v/>
       </c>
+      <c r="M22" s="9" t="n">
+        <v>230.1</v>
+      </c>
+      <c r="N22" s="9">
+        <f>IF(M22="","",D22*M22)</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1760,6 +1952,13 @@
         <f>IF(J23="","",D23*J23)</f>
         <v/>
       </c>
+      <c r="M23" s="4" t="n">
+        <v>247.8</v>
+      </c>
+      <c r="N23" s="4">
+        <f>IF(M23="","",D23*M23)</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
@@ -1803,6 +2002,13 @@
         <f>IF(J24="","",D24*J24)</f>
         <v/>
       </c>
+      <c r="M24" s="9" t="n">
+        <v>247.8</v>
+      </c>
+      <c r="N24" s="9">
+        <f>IF(M24="","",D24*M24)</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1846,6 +2052,11 @@
         <f>IF(J25="","",D25*J25)</f>
         <v/>
       </c>
+      <c r="M25" s="4" t="n"/>
+      <c r="N25" s="4">
+        <f>IF(M25="","",D25*M25)</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
@@ -1889,6 +2100,13 @@
         <f>IF(J26="","",D26*J26)</f>
         <v/>
       </c>
+      <c r="M26" s="9" t="n">
+        <v>247.8</v>
+      </c>
+      <c r="N26" s="9">
+        <f>IF(M26="","",D26*M26)</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1934,6 +2152,13 @@
         <f>IF(J27="","",D27*J27)</f>
         <v/>
       </c>
+      <c r="M27" s="4" t="n">
+        <v>247.8</v>
+      </c>
+      <c r="N27" s="4">
+        <f>IF(M27="","",D27*M27)</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
@@ -1979,6 +2204,13 @@
         <f>IF(J28="","",D28*J28)</f>
         <v/>
       </c>
+      <c r="M28" s="9" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="N28" s="9">
+        <f>IF(M28="","",D28*M28)</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2022,6 +2254,11 @@
         <f>IF(J29="","",D29*J29)</f>
         <v/>
       </c>
+      <c r="M29" s="4" t="n"/>
+      <c r="N29" s="4">
+        <f>IF(M29="","",D29*M29)</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
@@ -2063,6 +2300,11 @@
       </c>
       <c r="L30" s="9">
         <f>IF(J30="","",D30*J30)</f>
+        <v/>
+      </c>
+      <c r="M30" s="9" t="n"/>
+      <c r="N30" s="9">
+        <f>IF(M30="","",D30*M30)</f>
         <v/>
       </c>
     </row>
@@ -2107,6 +2349,11 @@
         <f>SUM(L3:L30)</f>
         <v/>
       </c>
+      <c r="M31" s="5" t="inlineStr"/>
+      <c r="N31" s="6">
+        <f>SUM(N3:N30)</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2118,6 +2365,19 @@
       <c r="C32" t="inlineStr"/>
       <c r="D32">
         <f>SUMIF(J3:J30,"",D3:D30)</f>
+        <v/>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32">
+        <f>SUMIF(M3:M30,"",D3:D30)</f>
         <v/>
       </c>
     </row>
@@ -2132,7 +2392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2147,6 +2407,8 @@
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="30" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2217,6 +2479,16 @@
           <t>Cost - new pigs (USD)</t>
         </is>
       </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>Rate - unrated pigs at Pin (USD)</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>Cost - new pigs, unrated at Pin rate (USD)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2262,6 +2534,13 @@
         <f>IF(J3="","",D3*J3)</f>
         <v/>
       </c>
+      <c r="M3" s="4" t="n">
+        <v>118</v>
+      </c>
+      <c r="N3" s="4">
+        <f>IF(M3="","",D3*M3)</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
@@ -2307,6 +2586,13 @@
         <f>IF(J4="","",D4*J4)</f>
         <v/>
       </c>
+      <c r="M4" s="9" t="n">
+        <v>118</v>
+      </c>
+      <c r="N4" s="9">
+        <f>IF(M4="","",D4*M4)</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2352,6 +2638,13 @@
         <f>IF(J5="","",D5*J5)</f>
         <v/>
       </c>
+      <c r="M5" s="4" t="n">
+        <v>129.8</v>
+      </c>
+      <c r="N5" s="4">
+        <f>IF(M5="","",D5*M5)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
@@ -2395,6 +2688,13 @@
         <f>IF(J6="","",D6*J6)</f>
         <v/>
       </c>
+      <c r="M6" s="9" t="n">
+        <v>129.8</v>
+      </c>
+      <c r="N6" s="9">
+        <f>IF(M6="","",D6*M6)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2438,6 +2738,11 @@
         <f>IF(J7="","",D7*J7)</f>
         <v/>
       </c>
+      <c r="M7" s="4" t="n"/>
+      <c r="N7" s="4">
+        <f>IF(M7="","",D7*M7)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
@@ -2481,6 +2786,13 @@
         <f>IF(J8="","",D8*J8)</f>
         <v/>
       </c>
+      <c r="M8" s="9" t="n">
+        <v>129.8</v>
+      </c>
+      <c r="N8" s="9">
+        <f>IF(M8="","",D8*M8)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2526,6 +2838,13 @@
         <f>IF(J9="","",D9*J9)</f>
         <v/>
       </c>
+      <c r="M9" s="4" t="n">
+        <v>129.8</v>
+      </c>
+      <c r="N9" s="4">
+        <f>IF(M9="","",D9*M9)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
@@ -2569,6 +2888,11 @@
         <f>IF(J10="","",D10*J10)</f>
         <v/>
       </c>
+      <c r="M10" s="9" t="n"/>
+      <c r="N10" s="9">
+        <f>IF(M10="","",D10*M10)</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2610,6 +2934,11 @@
       </c>
       <c r="L11" s="4">
         <f>IF(J11="","",D11*J11)</f>
+        <v/>
+      </c>
+      <c r="M11" s="4" t="n"/>
+      <c r="N11" s="4">
+        <f>IF(M11="","",D11*M11)</f>
         <v/>
       </c>
     </row>
@@ -2654,6 +2983,11 @@
         <f>SUM(L3:L11)</f>
         <v/>
       </c>
+      <c r="M12" s="5" t="inlineStr"/>
+      <c r="N12" s="6">
+        <f>SUM(N3:N11)</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2665,6 +2999,19 @@
       <c r="C13" t="inlineStr"/>
       <c r="D13">
         <f>SUMIF(J3:J11,"",D3:D11)</f>
+        <v/>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13">
+        <f>SUMIF(M3:M11,"",D3:D11)</f>
         <v/>
       </c>
     </row>
@@ -2679,7 +3026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:N49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2694,6 +3041,8 @@
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="30" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2764,6 +3113,16 @@
           <t>Cost - new pigs (USD)</t>
         </is>
       </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>Rate - unrated pigs at Pin (USD)</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>Cost - new pigs, unrated at Pin rate (USD)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2807,6 +3166,11 @@
         <f>IF(J3="","",D3*J3)</f>
         <v/>
       </c>
+      <c r="M3" s="4" t="n"/>
+      <c r="N3" s="4">
+        <f>IF(M3="","",D3*M3)</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
@@ -2850,6 +3214,11 @@
         <f>IF(J4="","",D4*J4)</f>
         <v/>
       </c>
+      <c r="M4" s="9" t="n"/>
+      <c r="N4" s="9">
+        <f>IF(M4="","",D4*M4)</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2893,6 +3262,11 @@
         <f>IF(J5="","",D5*J5)</f>
         <v/>
       </c>
+      <c r="M5" s="4" t="n"/>
+      <c r="N5" s="4">
+        <f>IF(M5="","",D5*M5)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
@@ -2936,6 +3310,11 @@
         <f>IF(J6="","",D6*J6)</f>
         <v/>
       </c>
+      <c r="M6" s="9" t="n"/>
+      <c r="N6" s="9">
+        <f>IF(M6="","",D6*M6)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2979,6 +3358,11 @@
         <f>IF(J7="","",D7*J7)</f>
         <v/>
       </c>
+      <c r="M7" s="4" t="n"/>
+      <c r="N7" s="4">
+        <f>IF(M7="","",D7*M7)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
@@ -3022,6 +3406,13 @@
         <f>IF(J8="","",D8*J8)</f>
         <v/>
       </c>
+      <c r="M8" s="9" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="N8" s="9">
+        <f>IF(M8="","",D8*M8)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3067,6 +3458,13 @@
         <f>IF(J9="","",D9*J9)</f>
         <v/>
       </c>
+      <c r="M9" s="4" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="N9" s="4">
+        <f>IF(M9="","",D9*M9)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
@@ -3112,6 +3510,13 @@
         <f>IF(J10="","",D10*J10)</f>
         <v/>
       </c>
+      <c r="M10" s="9" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="N10" s="9">
+        <f>IF(M10="","",D10*M10)</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3157,6 +3562,13 @@
         <f>IF(J11="","",D11*J11)</f>
         <v/>
       </c>
+      <c r="M11" s="4" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="N11" s="4">
+        <f>IF(M11="","",D11*M11)</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
@@ -3200,6 +3612,13 @@
         <f>IF(J12="","",D12*J12)</f>
         <v/>
       </c>
+      <c r="M12" s="9" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="N12" s="9">
+        <f>IF(M12="","",D12*M12)</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3245,6 +3664,13 @@
         <f>IF(J13="","",D13*J13)</f>
         <v/>
       </c>
+      <c r="M13" s="4" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="N13" s="4">
+        <f>IF(M13="","",D13*M13)</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
@@ -3288,6 +3714,11 @@
         <f>IF(J14="","",D14*J14)</f>
         <v/>
       </c>
+      <c r="M14" s="9" t="n"/>
+      <c r="N14" s="9">
+        <f>IF(M14="","",D14*M14)</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3331,6 +3762,11 @@
         <f>IF(J15="","",D15*J15)</f>
         <v/>
       </c>
+      <c r="M15" s="4" t="n"/>
+      <c r="N15" s="4">
+        <f>IF(M15="","",D15*M15)</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
@@ -3374,6 +3810,11 @@
         <f>IF(J16="","",D16*J16)</f>
         <v/>
       </c>
+      <c r="M16" s="9" t="n"/>
+      <c r="N16" s="9">
+        <f>IF(M16="","",D16*M16)</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3419,6 +3860,13 @@
         <f>IF(J17="","",D17*J17)</f>
         <v/>
       </c>
+      <c r="M17" s="4" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="N17" s="4">
+        <f>IF(M17="","",D17*M17)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
@@ -3464,6 +3912,13 @@
         <f>IF(J18="","",D18*J18)</f>
         <v/>
       </c>
+      <c r="M18" s="9" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="N18" s="9">
+        <f>IF(M18="","",D18*M18)</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3507,6 +3962,13 @@
         <f>IF(J19="","",D19*J19)</f>
         <v/>
       </c>
+      <c r="M19" s="4" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="N19" s="4">
+        <f>IF(M19="","",D19*M19)</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
@@ -3552,6 +4014,13 @@
         <f>IF(J20="","",D20*J20)</f>
         <v/>
       </c>
+      <c r="M20" s="9" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="N20" s="9">
+        <f>IF(M20="","",D20*M20)</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3595,6 +4064,11 @@
         <f>IF(J21="","",D21*J21)</f>
         <v/>
       </c>
+      <c r="M21" s="4" t="n"/>
+      <c r="N21" s="4">
+        <f>IF(M21="","",D21*M21)</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
@@ -3638,6 +4112,11 @@
         <f>IF(J22="","",D22*J22)</f>
         <v/>
       </c>
+      <c r="M22" s="9" t="n"/>
+      <c r="N22" s="9">
+        <f>IF(M22="","",D22*M22)</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3681,6 +4160,11 @@
         <f>IF(J23="","",D23*J23)</f>
         <v/>
       </c>
+      <c r="M23" s="4" t="n"/>
+      <c r="N23" s="4">
+        <f>IF(M23="","",D23*M23)</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
@@ -3724,6 +4208,11 @@
         <f>IF(J24="","",D24*J24)</f>
         <v/>
       </c>
+      <c r="M24" s="9" t="n"/>
+      <c r="N24" s="9">
+        <f>IF(M24="","",D24*M24)</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3769,6 +4258,13 @@
         <f>IF(J25="","",D25*J25)</f>
         <v/>
       </c>
+      <c r="M25" s="4" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="N25" s="4">
+        <f>IF(M25="","",D25*M25)</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
@@ -3814,6 +4310,13 @@
         <f>IF(J26="","",D26*J26)</f>
         <v/>
       </c>
+      <c r="M26" s="9" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="N26" s="9">
+        <f>IF(M26="","",D26*M26)</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3857,6 +4360,13 @@
         <f>IF(J27="","",D27*J27)</f>
         <v/>
       </c>
+      <c r="M27" s="4" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="N27" s="4">
+        <f>IF(M27="","",D27*M27)</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
@@ -3902,6 +4412,13 @@
         <f>IF(J28="","",D28*J28)</f>
         <v/>
       </c>
+      <c r="M28" s="9" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="N28" s="9">
+        <f>IF(M28="","",D28*M28)</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3945,6 +4462,11 @@
         <f>IF(J29="","",D29*J29)</f>
         <v/>
       </c>
+      <c r="M29" s="4" t="n"/>
+      <c r="N29" s="4">
+        <f>IF(M29="","",D29*M29)</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
@@ -3990,6 +4512,13 @@
         <f>IF(J30="","",D30*J30)</f>
         <v/>
       </c>
+      <c r="M30" s="9" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="N30" s="9">
+        <f>IF(M30="","",D30*M30)</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4033,6 +4562,11 @@
         <f>IF(J31="","",D31*J31)</f>
         <v/>
       </c>
+      <c r="M31" s="4" t="n"/>
+      <c r="N31" s="4">
+        <f>IF(M31="","",D31*M31)</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
@@ -4076,6 +4610,11 @@
         <f>IF(J32="","",D32*J32)</f>
         <v/>
       </c>
+      <c r="M32" s="9" t="n"/>
+      <c r="N32" s="9">
+        <f>IF(M32="","",D32*M32)</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4121,6 +4660,13 @@
         <f>IF(J33="","",D33*J33)</f>
         <v/>
       </c>
+      <c r="M33" s="4" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="N33" s="4">
+        <f>IF(M33="","",D33*M33)</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
@@ -4164,6 +4710,13 @@
         <f>IF(J34="","",D34*J34)</f>
         <v/>
       </c>
+      <c r="M34" s="9" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="N34" s="9">
+        <f>IF(M34="","",D34*M34)</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4209,6 +4762,13 @@
         <f>IF(J35="","",D35*J35)</f>
         <v/>
       </c>
+      <c r="M35" s="4" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="N35" s="4">
+        <f>IF(M35="","",D35*M35)</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
@@ -4252,6 +4812,11 @@
         <f>IF(J36="","",D36*J36)</f>
         <v/>
       </c>
+      <c r="M36" s="9" t="n"/>
+      <c r="N36" s="9">
+        <f>IF(M36="","",D36*M36)</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4295,6 +4860,11 @@
         <f>IF(J37="","",D37*J37)</f>
         <v/>
       </c>
+      <c r="M37" s="4" t="n"/>
+      <c r="N37" s="4">
+        <f>IF(M37="","",D37*M37)</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
@@ -4338,6 +4908,11 @@
         <f>IF(J38="","",D38*J38)</f>
         <v/>
       </c>
+      <c r="M38" s="9" t="n"/>
+      <c r="N38" s="9">
+        <f>IF(M38="","",D38*M38)</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4383,6 +4958,13 @@
         <f>IF(J39="","",D39*J39)</f>
         <v/>
       </c>
+      <c r="M39" s="4" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="N39" s="4">
+        <f>IF(M39="","",D39*M39)</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
@@ -4426,6 +5008,11 @@
         <f>IF(J40="","",D40*J40)</f>
         <v/>
       </c>
+      <c r="M40" s="9" t="n"/>
+      <c r="N40" s="9">
+        <f>IF(M40="","",D40*M40)</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4471,6 +5058,13 @@
         <f>IF(J41="","",D41*J41)</f>
         <v/>
       </c>
+      <c r="M41" s="4" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="N41" s="4">
+        <f>IF(M41="","",D41*M41)</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
@@ -4514,6 +5108,11 @@
         <f>IF(J42="","",D42*J42)</f>
         <v/>
       </c>
+      <c r="M42" s="9" t="n"/>
+      <c r="N42" s="9">
+        <f>IF(M42="","",D42*M42)</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -4559,6 +5158,13 @@
         <f>IF(J43="","",D43*J43)</f>
         <v/>
       </c>
+      <c r="M43" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="N43" s="4">
+        <f>IF(M43="","",D43*M43)</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="8" t="inlineStr">
@@ -4604,6 +5210,13 @@
         <f>IF(J44="","",D44*J44)</f>
         <v/>
       </c>
+      <c r="M44" s="9" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="N44" s="9">
+        <f>IF(M44="","",D44*M44)</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -4649,6 +5262,13 @@
         <f>IF(J45="","",D45*J45)</f>
         <v/>
       </c>
+      <c r="M45" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="N45" s="4">
+        <f>IF(M45="","",D45*M45)</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
@@ -4692,6 +5312,11 @@
         <f>IF(J46="","",D46*J46)</f>
         <v/>
       </c>
+      <c r="M46" s="9" t="n"/>
+      <c r="N46" s="9">
+        <f>IF(M46="","",D46*M46)</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4733,6 +5358,11 @@
       </c>
       <c r="L47" s="4">
         <f>IF(J47="","",D47*J47)</f>
+        <v/>
+      </c>
+      <c r="M47" s="4" t="n"/>
+      <c r="N47" s="4">
+        <f>IF(M47="","",D47*M47)</f>
         <v/>
       </c>
     </row>
@@ -4777,6 +5407,11 @@
         <f>SUM(L3:L47)</f>
         <v/>
       </c>
+      <c r="M48" s="5" t="inlineStr"/>
+      <c r="N48" s="6">
+        <f>SUM(N3:N47)</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -4788,6 +5423,19 @@
       <c r="C49" t="inlineStr"/>
       <c r="D49">
         <f>SUMIF(J3:J47,"",D3:D47)</f>
+        <v/>
+      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49">
+        <f>SUMIF(M3:M47,"",D3:D47)</f>
         <v/>
       </c>
     </row>
@@ -4802,7 +5450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:N40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4817,6 +5465,8 @@
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="30" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4887,6 +5537,16 @@
           <t>Cost - new pigs (USD)</t>
         </is>
       </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>Rate - unrated pigs at Pin (USD)</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>Cost - new pigs, unrated at Pin rate (USD)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4932,6 +5592,13 @@
         <f>IF(J3="","",D3*J3)</f>
         <v/>
       </c>
+      <c r="M3" s="4" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="N3" s="4">
+        <f>IF(M3="","",D3*M3)</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
@@ -4977,6 +5644,13 @@
         <f>IF(J4="","",D4*J4)</f>
         <v/>
       </c>
+      <c r="M4" s="9" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="N4" s="9">
+        <f>IF(M4="","",D4*M4)</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5020,6 +5694,11 @@
         <f>IF(J5="","",D5*J5)</f>
         <v/>
       </c>
+      <c r="M5" s="4" t="n"/>
+      <c r="N5" s="4">
+        <f>IF(M5="","",D5*M5)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
@@ -5065,6 +5744,13 @@
         <f>IF(J6="","",D6*J6)</f>
         <v/>
       </c>
+      <c r="M6" s="9" t="n">
+        <v>53.1</v>
+      </c>
+      <c r="N6" s="9">
+        <f>IF(M6="","",D6*M6)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -5110,6 +5796,13 @@
         <f>IF(J7="","",D7*J7)</f>
         <v/>
       </c>
+      <c r="M7" s="4" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="N7" s="4">
+        <f>IF(M7="","",D7*M7)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
@@ -5155,6 +5848,13 @@
         <f>IF(J8="","",D8*J8)</f>
         <v/>
       </c>
+      <c r="M8" s="9" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="N8" s="9">
+        <f>IF(M8="","",D8*M8)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5200,6 +5900,13 @@
         <f>IF(J9="","",D9*J9)</f>
         <v/>
       </c>
+      <c r="M9" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="N9" s="4">
+        <f>IF(M9="","",D9*M9)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
@@ -5245,6 +5952,13 @@
         <f>IF(J10="","",D10*J10)</f>
         <v/>
       </c>
+      <c r="M10" s="9" t="n">
+        <v>59</v>
+      </c>
+      <c r="N10" s="9">
+        <f>IF(M10="","",D10*M10)</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5288,6 +6002,11 @@
         <f>IF(J11="","",D11*J11)</f>
         <v/>
       </c>
+      <c r="M11" s="4" t="n"/>
+      <c r="N11" s="4">
+        <f>IF(M11="","",D11*M11)</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
@@ -5333,6 +6052,13 @@
         <f>IF(J12="","",D12*J12)</f>
         <v/>
       </c>
+      <c r="M12" s="9" t="n">
+        <v>59</v>
+      </c>
+      <c r="N12" s="9">
+        <f>IF(M12="","",D12*M12)</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5378,6 +6104,13 @@
         <f>IF(J13="","",D13*J13)</f>
         <v/>
       </c>
+      <c r="M13" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="N13" s="4">
+        <f>IF(M13="","",D13*M13)</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
@@ -5423,6 +6156,13 @@
         <f>IF(J14="","",D14*J14)</f>
         <v/>
       </c>
+      <c r="M14" s="9" t="n">
+        <v>64.90000000000001</v>
+      </c>
+      <c r="N14" s="9">
+        <f>IF(M14="","",D14*M14)</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5468,6 +6208,13 @@
         <f>IF(J15="","",D15*J15)</f>
         <v/>
       </c>
+      <c r="M15" s="4" t="n">
+        <v>64.90000000000001</v>
+      </c>
+      <c r="N15" s="4">
+        <f>IF(M15="","",D15*M15)</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
@@ -5511,6 +6258,11 @@
         <f>IF(J16="","",D16*J16)</f>
         <v/>
       </c>
+      <c r="M16" s="9" t="n"/>
+      <c r="N16" s="9">
+        <f>IF(M16="","",D16*M16)</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5554,6 +6306,11 @@
         <f>IF(J17="","",D17*J17)</f>
         <v/>
       </c>
+      <c r="M17" s="4" t="n"/>
+      <c r="N17" s="4">
+        <f>IF(M17="","",D17*M17)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
@@ -5597,6 +6354,11 @@
         <f>IF(J18="","",D18*J18)</f>
         <v/>
       </c>
+      <c r="M18" s="9" t="n"/>
+      <c r="N18" s="9">
+        <f>IF(M18="","",D18*M18)</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5642,6 +6404,13 @@
         <f>IF(J19="","",D19*J19)</f>
         <v/>
       </c>
+      <c r="M19" s="4" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="N19" s="4">
+        <f>IF(M19="","",D19*M19)</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
@@ -5687,6 +6456,13 @@
         <f>IF(J20="","",D20*J20)</f>
         <v/>
       </c>
+      <c r="M20" s="9" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="N20" s="9">
+        <f>IF(M20="","",D20*M20)</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5730,6 +6506,13 @@
         <f>IF(J21="","",D21*J21)</f>
         <v/>
       </c>
+      <c r="M21" s="4" t="n">
+        <v>118</v>
+      </c>
+      <c r="N21" s="4">
+        <f>IF(M21="","",D21*M21)</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
@@ -5775,6 +6558,13 @@
         <f>IF(J22="","",D22*J22)</f>
         <v/>
       </c>
+      <c r="M22" s="9" t="n">
+        <v>118</v>
+      </c>
+      <c r="N22" s="9">
+        <f>IF(M22="","",D22*M22)</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5820,6 +6610,13 @@
         <f>IF(J23="","",D23*J23)</f>
         <v/>
       </c>
+      <c r="M23" s="4" t="n">
+        <v>129.8</v>
+      </c>
+      <c r="N23" s="4">
+        <f>IF(M23="","",D23*M23)</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
@@ -5863,6 +6660,11 @@
         <f>IF(J24="","",D24*J24)</f>
         <v/>
       </c>
+      <c r="M24" s="9" t="n"/>
+      <c r="N24" s="9">
+        <f>IF(M24="","",D24*M24)</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5908,6 +6710,13 @@
         <f>IF(J25="","",D25*J25)</f>
         <v/>
       </c>
+      <c r="M25" s="4" t="n">
+        <v>129.8</v>
+      </c>
+      <c r="N25" s="4">
+        <f>IF(M25="","",D25*M25)</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
@@ -5953,6 +6762,13 @@
         <f>IF(J26="","",D26*J26)</f>
         <v/>
       </c>
+      <c r="M26" s="9" t="n">
+        <v>230.1</v>
+      </c>
+      <c r="N26" s="9">
+        <f>IF(M26="","",D26*M26)</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5996,6 +6812,11 @@
         <f>IF(J27="","",D27*J27)</f>
         <v/>
       </c>
+      <c r="M27" s="4" t="n"/>
+      <c r="N27" s="4">
+        <f>IF(M27="","",D27*M27)</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
@@ -6041,6 +6862,13 @@
         <f>IF(J28="","",D28*J28)</f>
         <v/>
       </c>
+      <c r="M28" s="9" t="n">
+        <v>247.8</v>
+      </c>
+      <c r="N28" s="9">
+        <f>IF(M28="","",D28*M28)</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -6086,6 +6914,13 @@
         <f>IF(J29="","",D29*J29)</f>
         <v/>
       </c>
+      <c r="M29" s="4" t="n">
+        <v>247.8</v>
+      </c>
+      <c r="N29" s="4">
+        <f>IF(M29="","",D29*M29)</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
@@ -6131,6 +6966,13 @@
         <f>IF(J30="","",D30*J30)</f>
         <v/>
       </c>
+      <c r="M30" s="9" t="n">
+        <v>483.8</v>
+      </c>
+      <c r="N30" s="9">
+        <f>IF(M30="","",D30*M30)</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -6176,6 +7018,13 @@
         <f>IF(J31="","",D31*J31)</f>
         <v/>
       </c>
+      <c r="M31" s="4" t="n">
+        <v>483.8</v>
+      </c>
+      <c r="N31" s="4">
+        <f>IF(M31="","",D31*M31)</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
@@ -6221,6 +7070,13 @@
         <f>IF(J32="","",D32*J32)</f>
         <v/>
       </c>
+      <c r="M32" s="9" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="N32" s="9">
+        <f>IF(M32="","",D32*M32)</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -6264,6 +7120,11 @@
         <f>IF(J33="","",D33*J33)</f>
         <v/>
       </c>
+      <c r="M33" s="4" t="n"/>
+      <c r="N33" s="4">
+        <f>IF(M33="","",D33*M33)</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
@@ -6309,6 +7170,13 @@
         <f>IF(J34="","",D34*J34)</f>
         <v/>
       </c>
+      <c r="M34" s="9" t="n">
+        <v>826</v>
+      </c>
+      <c r="N34" s="9">
+        <f>IF(M34="","",D34*M34)</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -6354,6 +7222,13 @@
         <f>IF(J35="","",D35*J35)</f>
         <v/>
       </c>
+      <c r="M35" s="4" t="n">
+        <v>826</v>
+      </c>
+      <c r="N35" s="4">
+        <f>IF(M35="","",D35*M35)</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
@@ -6397,6 +7272,11 @@
         <f>IF(J36="","",D36*J36)</f>
         <v/>
       </c>
+      <c r="M36" s="9" t="n"/>
+      <c r="N36" s="9">
+        <f>IF(M36="","",D36*M36)</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -6440,6 +7320,11 @@
         <f>IF(J37="","",D37*J37)</f>
         <v/>
       </c>
+      <c r="M37" s="4" t="n"/>
+      <c r="N37" s="4">
+        <f>IF(M37="","",D37*M37)</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
@@ -6481,6 +7366,11 @@
       </c>
       <c r="L38" s="9">
         <f>IF(J38="","",D38*J38)</f>
+        <v/>
+      </c>
+      <c r="M38" s="9" t="n"/>
+      <c r="N38" s="9">
+        <f>IF(M38="","",D38*M38)</f>
         <v/>
       </c>
     </row>
@@ -6525,6 +7415,11 @@
         <f>SUM(L3:L38)</f>
         <v/>
       </c>
+      <c r="M39" s="5" t="inlineStr"/>
+      <c r="N39" s="6">
+        <f>SUM(N3:N38)</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -6536,6 +7431,19 @@
       <c r="C40" t="inlineStr"/>
       <c r="D40">
         <f>SUMIF(J3:J38,"",D3:D38)</f>
+        <v/>
+      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40">
+        <f>SUMIF(M3:M38,"",D3:D38)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
[Lane 1] USA26046 pig counts: unrated pigs priced as Pin (Jesse); single cost basis
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02-facilities/Cenovus/Lima-OH/USA26046-pig-counts.xlsx
+++ b/02-facilities/Cenovus/Lima-OH/USA26046-pig-counts.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -475,8 +475,6 @@
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -544,16 +542,6 @@
           <t>New pigs with no rate</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>Cost - new pigs, unrated at Pin rate (USD)</t>
-        </is>
-      </c>
-      <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t>New pigs still with no rate</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -590,14 +578,6 @@
         <f>'Crude'!D32</f>
         <v/>
       </c>
-      <c r="K5" s="4">
-        <f>'Crude'!N31</f>
-        <v/>
-      </c>
-      <c r="L5">
-        <f>'Crude'!N32</f>
-        <v/>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -634,14 +614,6 @@
         <f>'HDS'!D13</f>
         <v/>
       </c>
-      <c r="K6" s="4">
-        <f>'HDS'!N12</f>
-        <v/>
-      </c>
-      <c r="L6">
-        <f>'HDS'!N13</f>
-        <v/>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -678,14 +650,6 @@
         <f>'Coker'!D49</f>
         <v/>
       </c>
-      <c r="K7" s="4">
-        <f>'Coker'!N48</f>
-        <v/>
-      </c>
-      <c r="L7">
-        <f>'Coker'!N49</f>
-        <v/>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -722,14 +686,6 @@
         <f>'Vac'!D40</f>
         <v/>
       </c>
-      <c r="K8" s="4">
-        <f>'Vac'!N39</f>
-        <v/>
-      </c>
-      <c r="L8">
-        <f>'Vac'!N40</f>
-        <v/>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -773,26 +729,18 @@
         <f>SUM(J5:J8)</f>
         <v/>
       </c>
-      <c r="K9" s="6">
-        <f>SUM(K5:K8)</f>
-        <v/>
-      </c>
-      <c r="L9" s="5">
-        <f>SUM(L5:L8)</f>
-        <v/>
-      </c>
     </row>
     <row r="11" ht="60" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Costing: New pigs only, at the pigs.xlsx rate for the same size and type; used pigs are not costed (Jesse, 2026-10-02). Bolted and HR pigs without their own rate take the same-size Pin rate (pigs.xlsx prices Bolt and HR the same as Pin wherever it lists both); Foam takes the Gauge Foam rate. Sizes or types not on pigs.xlsx carry no rate and are counted in "New pigs with no rate". Second view (Jesse, 2026-10-02: admin may count them as Pin): rated pigs unchanged; unrated Pin/HR/FMJ/unclear pigs take the same-size Pin rate where pigs.xlsx has one. Foams, swabs and honeycomb are not repriced. Neither view is treated as the correct one.</t>
+          <t>Costing: New pigs only; used pigs are not costed (Jesse, 2026-10-02). Rates are from pigs.xlsx for the same size and type. Any pig without its own rate is priced as Pin at the same size (Jesse, 2026-10-02: "Unrated are priced as PIN"). Foam takes the Gauge Foam rate; foams, swabs and honeycomb are not repriced as Pin. Sizes not on pigs.xlsx at all carry no rate and are counted in "New pigs with no rate".</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A11:L11"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A11:J11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -804,7 +752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N32"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -817,10 +765,8 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -891,16 +837,6 @@
           <t>Cost - new pigs (USD)</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
-        <is>
-          <t>Rate - unrated pigs at Pin (USD)</t>
-        </is>
-      </c>
-      <c r="N2" s="3" t="inlineStr">
-        <is>
-          <t>Cost - new pigs, unrated at Pin rate (USD)</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -944,11 +880,6 @@
         <f>IF(J3="","",D3*J3)</f>
         <v/>
       </c>
-      <c r="M3" s="4" t="n"/>
-      <c r="N3" s="4">
-        <f>IF(M3="","",D3*M3)</f>
-        <v/>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
@@ -992,11 +923,6 @@
         <f>IF(J4="","",D4*J4)</f>
         <v/>
       </c>
-      <c r="M4" s="9" t="n"/>
-      <c r="N4" s="9">
-        <f>IF(M4="","",D4*M4)</f>
-        <v/>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1035,20 +961,13 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>pigs.xlsx Pin rate, same size</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L5" s="4">
         <f>IF(J5="","",D5*J5)</f>
         <v/>
       </c>
-      <c r="M5" s="4" t="n">
-        <v>118</v>
-      </c>
-      <c r="N5" s="4">
-        <f>IF(M5="","",D5*M5)</f>
-        <v/>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
@@ -1094,13 +1013,6 @@
         <f>IF(J6="","",D6*J6)</f>
         <v/>
       </c>
-      <c r="M6" s="9" t="n">
-        <v>49.6</v>
-      </c>
-      <c r="N6" s="9">
-        <f>IF(M6="","",D6*M6)</f>
-        <v/>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1146,13 +1058,6 @@
         <f>IF(J7="","",D7*J7)</f>
         <v/>
       </c>
-      <c r="M7" s="4" t="n">
-        <v>49.6</v>
-      </c>
-      <c r="N7" s="4">
-        <f>IF(M7="","",D7*M7)</f>
-        <v/>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
@@ -1186,23 +1091,18 @@
       <c r="I8" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J8" s="9" t="n"/>
+      <c r="J8" s="9" t="n">
+        <v>118</v>
+      </c>
       <c r="K8" s="8" t="inlineStr">
         <is>
-          <t>no rate (type not on pigs.xlsx)</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L8" s="9">
         <f>IF(J8="","",D8*J8)</f>
         <v/>
       </c>
-      <c r="M8" s="9" t="n">
-        <v>118</v>
-      </c>
-      <c r="N8" s="9">
-        <f>IF(M8="","",D8*M8)</f>
-        <v/>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1248,13 +1148,6 @@
         <f>IF(J9="","",D9*J9)</f>
         <v/>
       </c>
-      <c r="M9" s="4" t="n">
-        <v>118</v>
-      </c>
-      <c r="N9" s="4">
-        <f>IF(M9="","",D9*M9)</f>
-        <v/>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
@@ -1293,20 +1186,13 @@
       </c>
       <c r="K10" s="8" t="inlineStr">
         <is>
-          <t>pigs.xlsx Pin rate, same size</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L10" s="9">
         <f>IF(J10="","",D10*J10)</f>
         <v/>
       </c>
-      <c r="M10" s="9" t="n">
-        <v>129.8</v>
-      </c>
-      <c r="N10" s="9">
-        <f>IF(M10="","",D10*M10)</f>
-        <v/>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1352,13 +1238,6 @@
         <f>IF(J11="","",D11*J11)</f>
         <v/>
       </c>
-      <c r="M11" s="4" t="n">
-        <v>129.8</v>
-      </c>
-      <c r="N11" s="4">
-        <f>IF(M11="","",D11*M11)</f>
-        <v/>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
@@ -1392,23 +1271,18 @@
       <c r="I12" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J12" s="9" t="n"/>
+      <c r="J12" s="9" t="n">
+        <v>129.8</v>
+      </c>
       <c r="K12" s="8" t="inlineStr">
         <is>
-          <t>no rate (type not on pigs.xlsx)</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L12" s="9">
         <f>IF(J12="","",D12*J12)</f>
         <v/>
       </c>
-      <c r="M12" s="9" t="n">
-        <v>129.8</v>
-      </c>
-      <c r="N12" s="9">
-        <f>IF(M12="","",D12*M12)</f>
-        <v/>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1442,23 +1316,18 @@
       <c r="I13" t="n">
         <v>0</v>
       </c>
-      <c r="J13" s="4" t="n"/>
+      <c r="J13" s="4" t="n">
+        <v>129.8</v>
+      </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>no rate (type not on pigs.xlsx)</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L13" s="4">
         <f>IF(J13="","",D13*J13)</f>
         <v/>
       </c>
-      <c r="M13" s="4" t="n">
-        <v>129.8</v>
-      </c>
-      <c r="N13" s="4">
-        <f>IF(M13="","",D13*M13)</f>
-        <v/>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
@@ -1504,13 +1373,6 @@
         <f>IF(J14="","",D14*J14)</f>
         <v/>
       </c>
-      <c r="M14" s="9" t="n">
-        <v>129.8</v>
-      </c>
-      <c r="N14" s="9">
-        <f>IF(M14="","",D14*M14)</f>
-        <v/>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1554,11 +1416,6 @@
         <f>IF(J15="","",D15*J15)</f>
         <v/>
       </c>
-      <c r="M15" s="4" t="n"/>
-      <c r="N15" s="4">
-        <f>IF(M15="","",D15*M15)</f>
-        <v/>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
@@ -1602,11 +1459,6 @@
         <f>IF(J16="","",D16*J16)</f>
         <v/>
       </c>
-      <c r="M16" s="9" t="n"/>
-      <c r="N16" s="9">
-        <f>IF(M16="","",D16*M16)</f>
-        <v/>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1643,18 +1495,13 @@
       <c r="J17" s="4" t="n"/>
       <c r="K17" t="inlineStr">
         <is>
-          <t>no rate (type not on pigs.xlsx)</t>
+          <t>no rate (size not on pigs.xlsx)</t>
         </is>
       </c>
       <c r="L17" s="4">
         <f>IF(J17="","",D17*J17)</f>
         <v/>
       </c>
-      <c r="M17" s="4" t="n"/>
-      <c r="N17" s="4">
-        <f>IF(M17="","",D17*M17)</f>
-        <v/>
-      </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
@@ -1698,11 +1545,6 @@
         <f>IF(J18="","",D18*J18)</f>
         <v/>
       </c>
-      <c r="M18" s="9" t="n"/>
-      <c r="N18" s="9">
-        <f>IF(M18="","",D18*M18)</f>
-        <v/>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1748,13 +1590,6 @@
         <f>IF(J19="","",D19*J19)</f>
         <v/>
       </c>
-      <c r="M19" s="4" t="n">
-        <v>230.1</v>
-      </c>
-      <c r="N19" s="4">
-        <f>IF(M19="","",D19*M19)</f>
-        <v/>
-      </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
@@ -1788,23 +1623,18 @@
       <c r="I20" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J20" s="9" t="n"/>
+      <c r="J20" s="9" t="n">
+        <v>230.1</v>
+      </c>
       <c r="K20" s="8" t="inlineStr">
         <is>
-          <t>no rate (type not on pigs.xlsx)</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L20" s="9">
         <f>IF(J20="","",D20*J20)</f>
         <v/>
       </c>
-      <c r="M20" s="9" t="n">
-        <v>230.1</v>
-      </c>
-      <c r="N20" s="9">
-        <f>IF(M20="","",D20*M20)</f>
-        <v/>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1838,23 +1668,18 @@
       <c r="I21" t="n">
         <v>0</v>
       </c>
-      <c r="J21" s="4" t="n"/>
+      <c r="J21" s="4" t="n">
+        <v>230.1</v>
+      </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>no rate (type not on pigs.xlsx)</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L21" s="4">
         <f>IF(J21="","",D21*J21)</f>
         <v/>
       </c>
-      <c r="M21" s="4" t="n">
-        <v>230.1</v>
-      </c>
-      <c r="N21" s="4">
-        <f>IF(M21="","",D21*M21)</f>
-        <v/>
-      </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
@@ -1900,13 +1725,6 @@
         <f>IF(J22="","",D22*J22)</f>
         <v/>
       </c>
-      <c r="M22" s="9" t="n">
-        <v>230.1</v>
-      </c>
-      <c r="N22" s="9">
-        <f>IF(M22="","",D22*M22)</f>
-        <v/>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1952,13 +1770,6 @@
         <f>IF(J23="","",D23*J23)</f>
         <v/>
       </c>
-      <c r="M23" s="4" t="n">
-        <v>247.8</v>
-      </c>
-      <c r="N23" s="4">
-        <f>IF(M23="","",D23*M23)</f>
-        <v/>
-      </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
@@ -1992,23 +1803,18 @@
       <c r="I24" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J24" s="9" t="n"/>
+      <c r="J24" s="9" t="n">
+        <v>247.8</v>
+      </c>
       <c r="K24" s="8" t="inlineStr">
         <is>
-          <t>no rate (type not on pigs.xlsx)</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L24" s="9">
         <f>IF(J24="","",D24*J24)</f>
         <v/>
       </c>
-      <c r="M24" s="9" t="n">
-        <v>247.8</v>
-      </c>
-      <c r="N24" s="9">
-        <f>IF(M24="","",D24*M24)</f>
-        <v/>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2052,11 +1858,6 @@
         <f>IF(J25="","",D25*J25)</f>
         <v/>
       </c>
-      <c r="M25" s="4" t="n"/>
-      <c r="N25" s="4">
-        <f>IF(M25="","",D25*M25)</f>
-        <v/>
-      </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
@@ -2090,23 +1891,18 @@
       <c r="I26" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J26" s="9" t="n"/>
+      <c r="J26" s="9" t="n">
+        <v>247.8</v>
+      </c>
       <c r="K26" s="8" t="inlineStr">
         <is>
-          <t>no rate (type not on pigs.xlsx)</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L26" s="9">
         <f>IF(J26="","",D26*J26)</f>
         <v/>
       </c>
-      <c r="M26" s="9" t="n">
-        <v>247.8</v>
-      </c>
-      <c r="N26" s="9">
-        <f>IF(M26="","",D26*M26)</f>
-        <v/>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2152,13 +1948,6 @@
         <f>IF(J27="","",D27*J27)</f>
         <v/>
       </c>
-      <c r="M27" s="4" t="n">
-        <v>247.8</v>
-      </c>
-      <c r="N27" s="4">
-        <f>IF(M27="","",D27*M27)</f>
-        <v/>
-      </c>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
@@ -2204,13 +1993,6 @@
         <f>IF(J28="","",D28*J28)</f>
         <v/>
       </c>
-      <c r="M28" s="9" t="n">
-        <v>16.1</v>
-      </c>
-      <c r="N28" s="9">
-        <f>IF(M28="","",D28*M28)</f>
-        <v/>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2254,11 +2036,6 @@
         <f>IF(J29="","",D29*J29)</f>
         <v/>
       </c>
-      <c r="M29" s="4" t="n"/>
-      <c r="N29" s="4">
-        <f>IF(M29="","",D29*M29)</f>
-        <v/>
-      </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
@@ -2300,11 +2077,6 @@
       </c>
       <c r="L30" s="9">
         <f>IF(J30="","",D30*J30)</f>
-        <v/>
-      </c>
-      <c r="M30" s="9" t="n"/>
-      <c r="N30" s="9">
-        <f>IF(M30="","",D30*M30)</f>
         <v/>
       </c>
     </row>
@@ -2349,11 +2121,6 @@
         <f>SUM(L3:L30)</f>
         <v/>
       </c>
-      <c r="M31" s="5" t="inlineStr"/>
-      <c r="N31" s="6">
-        <f>SUM(N3:N30)</f>
-        <v/>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2365,19 +2132,6 @@
       <c r="C32" t="inlineStr"/>
       <c r="D32">
         <f>SUMIF(J3:J30,"",D3:D30)</f>
-        <v/>
-      </c>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32">
-        <f>SUMIF(M3:M30,"",D3:D30)</f>
         <v/>
       </c>
     </row>
@@ -2392,7 +2146,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2405,10 +2159,8 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2479,16 +2231,6 @@
           <t>Cost - new pigs (USD)</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
-        <is>
-          <t>Rate - unrated pigs at Pin (USD)</t>
-        </is>
-      </c>
-      <c r="N2" s="3" t="inlineStr">
-        <is>
-          <t>Cost - new pigs, unrated at Pin rate (USD)</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2527,20 +2269,13 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>pigs.xlsx Pin rate, same size</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L3" s="4">
         <f>IF(J3="","",D3*J3)</f>
         <v/>
       </c>
-      <c r="M3" s="4" t="n">
-        <v>118</v>
-      </c>
-      <c r="N3" s="4">
-        <f>IF(M3="","",D3*M3)</f>
-        <v/>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
@@ -2586,13 +2321,6 @@
         <f>IF(J4="","",D4*J4)</f>
         <v/>
       </c>
-      <c r="M4" s="9" t="n">
-        <v>118</v>
-      </c>
-      <c r="N4" s="9">
-        <f>IF(M4="","",D4*M4)</f>
-        <v/>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2638,13 +2366,6 @@
         <f>IF(J5="","",D5*J5)</f>
         <v/>
       </c>
-      <c r="M5" s="4" t="n">
-        <v>129.8</v>
-      </c>
-      <c r="N5" s="4">
-        <f>IF(M5="","",D5*M5)</f>
-        <v/>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
@@ -2678,23 +2399,18 @@
       <c r="I6" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J6" s="9" t="n"/>
+      <c r="J6" s="9" t="n">
+        <v>129.8</v>
+      </c>
       <c r="K6" s="8" t="inlineStr">
         <is>
-          <t>no rate (type not on pigs.xlsx)</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L6" s="9">
         <f>IF(J6="","",D6*J6)</f>
         <v/>
       </c>
-      <c r="M6" s="9" t="n">
-        <v>129.8</v>
-      </c>
-      <c r="N6" s="9">
-        <f>IF(M6="","",D6*M6)</f>
-        <v/>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2738,11 +2454,6 @@
         <f>IF(J7="","",D7*J7)</f>
         <v/>
       </c>
-      <c r="M7" s="4" t="n"/>
-      <c r="N7" s="4">
-        <f>IF(M7="","",D7*M7)</f>
-        <v/>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
@@ -2776,23 +2487,18 @@
       <c r="I8" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J8" s="9" t="n"/>
+      <c r="J8" s="9" t="n">
+        <v>129.8</v>
+      </c>
       <c r="K8" s="8" t="inlineStr">
         <is>
-          <t>no rate (type not on pigs.xlsx)</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L8" s="9">
         <f>IF(J8="","",D8*J8)</f>
         <v/>
       </c>
-      <c r="M8" s="9" t="n">
-        <v>129.8</v>
-      </c>
-      <c r="N8" s="9">
-        <f>IF(M8="","",D8*M8)</f>
-        <v/>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2838,13 +2544,6 @@
         <f>IF(J9="","",D9*J9)</f>
         <v/>
       </c>
-      <c r="M9" s="4" t="n">
-        <v>129.8</v>
-      </c>
-      <c r="N9" s="4">
-        <f>IF(M9="","",D9*M9)</f>
-        <v/>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
@@ -2881,18 +2580,13 @@
       <c r="J10" s="9" t="n"/>
       <c r="K10" s="8" t="inlineStr">
         <is>
-          <t>no rate (type not on pigs.xlsx)</t>
+          <t>no rate (size not on pigs.xlsx)</t>
         </is>
       </c>
       <c r="L10" s="9">
         <f>IF(J10="","",D10*J10)</f>
         <v/>
       </c>
-      <c r="M10" s="9" t="n"/>
-      <c r="N10" s="9">
-        <f>IF(M10="","",D10*M10)</f>
-        <v/>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2934,11 +2628,6 @@
       </c>
       <c r="L11" s="4">
         <f>IF(J11="","",D11*J11)</f>
-        <v/>
-      </c>
-      <c r="M11" s="4" t="n"/>
-      <c r="N11" s="4">
-        <f>IF(M11="","",D11*M11)</f>
         <v/>
       </c>
     </row>
@@ -2983,11 +2672,6 @@
         <f>SUM(L3:L11)</f>
         <v/>
       </c>
-      <c r="M12" s="5" t="inlineStr"/>
-      <c r="N12" s="6">
-        <f>SUM(N3:N11)</f>
-        <v/>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2999,19 +2683,6 @@
       <c r="C13" t="inlineStr"/>
       <c r="D13">
         <f>SUMIF(J3:J11,"",D3:D11)</f>
-        <v/>
-      </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13">
-        <f>SUMIF(M3:M11,"",D3:D11)</f>
         <v/>
       </c>
     </row>
@@ -3026,7 +2697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N49"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3039,10 +2710,8 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3113,16 +2782,6 @@
           <t>Cost - new pigs (USD)</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
-        <is>
-          <t>Rate - unrated pigs at Pin (USD)</t>
-        </is>
-      </c>
-      <c r="N2" s="3" t="inlineStr">
-        <is>
-          <t>Cost - new pigs, unrated at Pin rate (USD)</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3166,11 +2825,6 @@
         <f>IF(J3="","",D3*J3)</f>
         <v/>
       </c>
-      <c r="M3" s="4" t="n"/>
-      <c r="N3" s="4">
-        <f>IF(M3="","",D3*M3)</f>
-        <v/>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
@@ -3214,11 +2868,6 @@
         <f>IF(J4="","",D4*J4)</f>
         <v/>
       </c>
-      <c r="M4" s="9" t="n"/>
-      <c r="N4" s="9">
-        <f>IF(M4="","",D4*M4)</f>
-        <v/>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3262,11 +2911,6 @@
         <f>IF(J5="","",D5*J5)</f>
         <v/>
       </c>
-      <c r="M5" s="4" t="n"/>
-      <c r="N5" s="4">
-        <f>IF(M5="","",D5*M5)</f>
-        <v/>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
@@ -3310,11 +2954,6 @@
         <f>IF(J6="","",D6*J6)</f>
         <v/>
       </c>
-      <c r="M6" s="9" t="n"/>
-      <c r="N6" s="9">
-        <f>IF(M6="","",D6*M6)</f>
-        <v/>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3358,11 +2997,6 @@
         <f>IF(J7="","",D7*J7)</f>
         <v/>
       </c>
-      <c r="M7" s="4" t="n"/>
-      <c r="N7" s="4">
-        <f>IF(M7="","",D7*M7)</f>
-        <v/>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
@@ -3396,23 +3030,18 @@
       <c r="I8" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J8" s="9" t="n"/>
+      <c r="J8" s="9" t="n">
+        <v>41.3</v>
+      </c>
       <c r="K8" s="8" t="inlineStr">
         <is>
-          <t>no rate (type not on pigs.xlsx)</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L8" s="9">
         <f>IF(J8="","",D8*J8)</f>
         <v/>
       </c>
-      <c r="M8" s="9" t="n">
-        <v>41.3</v>
-      </c>
-      <c r="N8" s="9">
-        <f>IF(M8="","",D8*M8)</f>
-        <v/>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3458,13 +3087,6 @@
         <f>IF(J9="","",D9*J9)</f>
         <v/>
       </c>
-      <c r="M9" s="4" t="n">
-        <v>41.3</v>
-      </c>
-      <c r="N9" s="4">
-        <f>IF(M9="","",D9*M9)</f>
-        <v/>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
@@ -3503,20 +3125,13 @@
       </c>
       <c r="K10" s="8" t="inlineStr">
         <is>
-          <t>pigs.xlsx Pin rate, same size</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L10" s="9">
         <f>IF(J10="","",D10*J10)</f>
         <v/>
       </c>
-      <c r="M10" s="9" t="n">
-        <v>41.3</v>
-      </c>
-      <c r="N10" s="9">
-        <f>IF(M10="","",D10*M10)</f>
-        <v/>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3555,20 +3170,13 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>pigs.xlsx Pin rate, same size</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L11" s="4">
         <f>IF(J11="","",D11*J11)</f>
         <v/>
       </c>
-      <c r="M11" s="4" t="n">
-        <v>41.3</v>
-      </c>
-      <c r="N11" s="4">
-        <f>IF(M11="","",D11*M11)</f>
-        <v/>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
@@ -3602,23 +3210,18 @@
       <c r="I12" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J12" s="9" t="n"/>
+      <c r="J12" s="9" t="n">
+        <v>41.3</v>
+      </c>
       <c r="K12" s="8" t="inlineStr">
         <is>
-          <t>no rate (type not on pigs.xlsx)</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L12" s="9">
         <f>IF(J12="","",D12*J12)</f>
         <v/>
       </c>
-      <c r="M12" s="9" t="n">
-        <v>41.3</v>
-      </c>
-      <c r="N12" s="9">
-        <f>IF(M12="","",D12*M12)</f>
-        <v/>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3664,13 +3267,6 @@
         <f>IF(J13="","",D13*J13)</f>
         <v/>
       </c>
-      <c r="M13" s="4" t="n">
-        <v>41.3</v>
-      </c>
-      <c r="N13" s="4">
-        <f>IF(M13="","",D13*M13)</f>
-        <v/>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
@@ -3714,11 +3310,6 @@
         <f>IF(J14="","",D14*J14)</f>
         <v/>
       </c>
-      <c r="M14" s="9" t="n"/>
-      <c r="N14" s="9">
-        <f>IF(M14="","",D14*M14)</f>
-        <v/>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3762,11 +3353,6 @@
         <f>IF(J15="","",D15*J15)</f>
         <v/>
       </c>
-      <c r="M15" s="4" t="n"/>
-      <c r="N15" s="4">
-        <f>IF(M15="","",D15*M15)</f>
-        <v/>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
@@ -3810,11 +3396,6 @@
         <f>IF(J16="","",D16*J16)</f>
         <v/>
       </c>
-      <c r="M16" s="9" t="n"/>
-      <c r="N16" s="9">
-        <f>IF(M16="","",D16*M16)</f>
-        <v/>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3853,20 +3434,13 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>pigs.xlsx Pin rate, same size</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L17" s="4">
         <f>IF(J17="","",D17*J17)</f>
         <v/>
       </c>
-      <c r="M17" s="4" t="n">
-        <v>47.2</v>
-      </c>
-      <c r="N17" s="4">
-        <f>IF(M17="","",D17*M17)</f>
-        <v/>
-      </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
@@ -3905,20 +3479,13 @@
       </c>
       <c r="K18" s="8" t="inlineStr">
         <is>
-          <t>pigs.xlsx Pin rate, same size</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L18" s="9">
         <f>IF(J18="","",D18*J18)</f>
         <v/>
       </c>
-      <c r="M18" s="9" t="n">
-        <v>47.2</v>
-      </c>
-      <c r="N18" s="9">
-        <f>IF(M18="","",D18*M18)</f>
-        <v/>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3952,23 +3519,18 @@
       <c r="I19" t="n">
         <v>0</v>
       </c>
-      <c r="J19" s="4" t="n"/>
+      <c r="J19" s="4" t="n">
+        <v>47.2</v>
+      </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>no rate (type not on pigs.xlsx)</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L19" s="4">
         <f>IF(J19="","",D19*J19)</f>
         <v/>
       </c>
-      <c r="M19" s="4" t="n">
-        <v>47.2</v>
-      </c>
-      <c r="N19" s="4">
-        <f>IF(M19="","",D19*M19)</f>
-        <v/>
-      </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
@@ -4014,13 +3576,6 @@
         <f>IF(J20="","",D20*J20)</f>
         <v/>
       </c>
-      <c r="M20" s="9" t="n">
-        <v>47.2</v>
-      </c>
-      <c r="N20" s="9">
-        <f>IF(M20="","",D20*M20)</f>
-        <v/>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4064,11 +3619,6 @@
         <f>IF(J21="","",D21*J21)</f>
         <v/>
       </c>
-      <c r="M21" s="4" t="n"/>
-      <c r="N21" s="4">
-        <f>IF(M21="","",D21*M21)</f>
-        <v/>
-      </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
@@ -4112,11 +3662,6 @@
         <f>IF(J22="","",D22*J22)</f>
         <v/>
       </c>
-      <c r="M22" s="9" t="n"/>
-      <c r="N22" s="9">
-        <f>IF(M22="","",D22*M22)</f>
-        <v/>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4153,18 +3698,13 @@
       <c r="J23" s="4" t="n"/>
       <c r="K23" t="inlineStr">
         <is>
-          <t>no rate (type not on pigs.xlsx)</t>
+          <t>no rate (size not on pigs.xlsx)</t>
         </is>
       </c>
       <c r="L23" s="4">
         <f>IF(J23="","",D23*J23)</f>
         <v/>
       </c>
-      <c r="M23" s="4" t="n"/>
-      <c r="N23" s="4">
-        <f>IF(M23="","",D23*M23)</f>
-        <v/>
-      </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
@@ -4208,11 +3748,6 @@
         <f>IF(J24="","",D24*J24)</f>
         <v/>
       </c>
-      <c r="M24" s="9" t="n"/>
-      <c r="N24" s="9">
-        <f>IF(M24="","",D24*M24)</f>
-        <v/>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4251,20 +3786,13 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>pigs.xlsx Pin rate, same size</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L25" s="4">
         <f>IF(J25="","",D25*J25)</f>
         <v/>
       </c>
-      <c r="M25" s="4" t="n">
-        <v>47.2</v>
-      </c>
-      <c r="N25" s="4">
-        <f>IF(M25="","",D25*M25)</f>
-        <v/>
-      </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
@@ -4303,20 +3831,13 @@
       </c>
       <c r="K26" s="8" t="inlineStr">
         <is>
-          <t>pigs.xlsx Pin rate, same size</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L26" s="9">
         <f>IF(J26="","",D26*J26)</f>
         <v/>
       </c>
-      <c r="M26" s="9" t="n">
-        <v>47.2</v>
-      </c>
-      <c r="N26" s="9">
-        <f>IF(M26="","",D26*M26)</f>
-        <v/>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4350,23 +3871,18 @@
       <c r="I27" t="n">
         <v>0</v>
       </c>
-      <c r="J27" s="4" t="n"/>
+      <c r="J27" s="4" t="n">
+        <v>47.2</v>
+      </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>no rate (type not on pigs.xlsx)</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L27" s="4">
         <f>IF(J27="","",D27*J27)</f>
         <v/>
       </c>
-      <c r="M27" s="4" t="n">
-        <v>47.2</v>
-      </c>
-      <c r="N27" s="4">
-        <f>IF(M27="","",D27*M27)</f>
-        <v/>
-      </c>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
@@ -4412,13 +3928,6 @@
         <f>IF(J28="","",D28*J28)</f>
         <v/>
       </c>
-      <c r="M28" s="9" t="n">
-        <v>47.2</v>
-      </c>
-      <c r="N28" s="9">
-        <f>IF(M28="","",D28*M28)</f>
-        <v/>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4462,11 +3971,6 @@
         <f>IF(J29="","",D29*J29)</f>
         <v/>
       </c>
-      <c r="M29" s="4" t="n"/>
-      <c r="N29" s="4">
-        <f>IF(M29="","",D29*M29)</f>
-        <v/>
-      </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
@@ -4505,20 +4009,13 @@
       </c>
       <c r="K30" s="8" t="inlineStr">
         <is>
-          <t>pigs.xlsx Pin rate, same size</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L30" s="9">
         <f>IF(J30="","",D30*J30)</f>
         <v/>
       </c>
-      <c r="M30" s="9" t="n">
-        <v>53.1</v>
-      </c>
-      <c r="N30" s="9">
-        <f>IF(M30="","",D30*M30)</f>
-        <v/>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4562,11 +4059,6 @@
         <f>IF(J31="","",D31*J31)</f>
         <v/>
       </c>
-      <c r="M31" s="4" t="n"/>
-      <c r="N31" s="4">
-        <f>IF(M31="","",D31*M31)</f>
-        <v/>
-      </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
@@ -4610,11 +4102,6 @@
         <f>IF(J32="","",D32*J32)</f>
         <v/>
       </c>
-      <c r="M32" s="9" t="n"/>
-      <c r="N32" s="9">
-        <f>IF(M32="","",D32*M32)</f>
-        <v/>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4653,20 +4140,13 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>pigs.xlsx Pin rate, same size</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L33" s="4">
         <f>IF(J33="","",D33*J33)</f>
         <v/>
       </c>
-      <c r="M33" s="4" t="n">
-        <v>53.1</v>
-      </c>
-      <c r="N33" s="4">
-        <f>IF(M33="","",D33*M33)</f>
-        <v/>
-      </c>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
@@ -4700,23 +4180,18 @@
       <c r="I34" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J34" s="9" t="n"/>
+      <c r="J34" s="9" t="n">
+        <v>53.1</v>
+      </c>
       <c r="K34" s="8" t="inlineStr">
         <is>
-          <t>no rate (type not on pigs.xlsx)</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L34" s="9">
         <f>IF(J34="","",D34*J34)</f>
         <v/>
       </c>
-      <c r="M34" s="9" t="n">
-        <v>53.1</v>
-      </c>
-      <c r="N34" s="9">
-        <f>IF(M34="","",D34*M34)</f>
-        <v/>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4762,13 +4237,6 @@
         <f>IF(J35="","",D35*J35)</f>
         <v/>
       </c>
-      <c r="M35" s="4" t="n">
-        <v>53.1</v>
-      </c>
-      <c r="N35" s="4">
-        <f>IF(M35="","",D35*M35)</f>
-        <v/>
-      </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
@@ -4812,11 +4280,6 @@
         <f>IF(J36="","",D36*J36)</f>
         <v/>
       </c>
-      <c r="M36" s="9" t="n"/>
-      <c r="N36" s="9">
-        <f>IF(M36="","",D36*M36)</f>
-        <v/>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4860,11 +4323,6 @@
         <f>IF(J37="","",D37*J37)</f>
         <v/>
       </c>
-      <c r="M37" s="4" t="n"/>
-      <c r="N37" s="4">
-        <f>IF(M37="","",D37*M37)</f>
-        <v/>
-      </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
@@ -4908,11 +4366,6 @@
         <f>IF(J38="","",D38*J38)</f>
         <v/>
       </c>
-      <c r="M38" s="9" t="n"/>
-      <c r="N38" s="9">
-        <f>IF(M38="","",D38*M38)</f>
-        <v/>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4951,20 +4404,13 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>pigs.xlsx Pin rate, same size</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L39" s="4">
         <f>IF(J39="","",D39*J39)</f>
         <v/>
       </c>
-      <c r="M39" s="4" t="n">
-        <v>53.1</v>
-      </c>
-      <c r="N39" s="4">
-        <f>IF(M39="","",D39*M39)</f>
-        <v/>
-      </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
@@ -5008,11 +4454,6 @@
         <f>IF(J40="","",D40*J40)</f>
         <v/>
       </c>
-      <c r="M40" s="9" t="n"/>
-      <c r="N40" s="9">
-        <f>IF(M40="","",D40*M40)</f>
-        <v/>
-      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -5058,13 +4499,6 @@
         <f>IF(J41="","",D41*J41)</f>
         <v/>
       </c>
-      <c r="M41" s="4" t="n">
-        <v>53.1</v>
-      </c>
-      <c r="N41" s="4">
-        <f>IF(M41="","",D41*M41)</f>
-        <v/>
-      </c>
     </row>
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
@@ -5108,11 +4542,6 @@
         <f>IF(J42="","",D42*J42)</f>
         <v/>
       </c>
-      <c r="M42" s="9" t="n"/>
-      <c r="N42" s="9">
-        <f>IF(M42="","",D42*M42)</f>
-        <v/>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -5151,20 +4580,13 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>pigs.xlsx Pin rate, same size</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L43" s="4">
         <f>IF(J43="","",D43*J43)</f>
         <v/>
       </c>
-      <c r="M43" s="4" t="n">
-        <v>59</v>
-      </c>
-      <c r="N43" s="4">
-        <f>IF(M43="","",D43*M43)</f>
-        <v/>
-      </c>
     </row>
     <row r="44">
       <c r="A44" s="8" t="inlineStr">
@@ -5210,13 +4632,6 @@
         <f>IF(J44="","",D44*J44)</f>
         <v/>
       </c>
-      <c r="M44" s="9" t="n">
-        <v>18.9</v>
-      </c>
-      <c r="N44" s="9">
-        <f>IF(M44="","",D44*M44)</f>
-        <v/>
-      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -5262,13 +4677,6 @@
         <f>IF(J45="","",D45*J45)</f>
         <v/>
       </c>
-      <c r="M45" s="4" t="n">
-        <v>59</v>
-      </c>
-      <c r="N45" s="4">
-        <f>IF(M45="","",D45*M45)</f>
-        <v/>
-      </c>
     </row>
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
@@ -5312,11 +4720,6 @@
         <f>IF(J46="","",D46*J46)</f>
         <v/>
       </c>
-      <c r="M46" s="9" t="n"/>
-      <c r="N46" s="9">
-        <f>IF(M46="","",D46*M46)</f>
-        <v/>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -5358,11 +4761,6 @@
       </c>
       <c r="L47" s="4">
         <f>IF(J47="","",D47*J47)</f>
-        <v/>
-      </c>
-      <c r="M47" s="4" t="n"/>
-      <c r="N47" s="4">
-        <f>IF(M47="","",D47*M47)</f>
         <v/>
       </c>
     </row>
@@ -5407,11 +4805,6 @@
         <f>SUM(L3:L47)</f>
         <v/>
       </c>
-      <c r="M48" s="5" t="inlineStr"/>
-      <c r="N48" s="6">
-        <f>SUM(N3:N47)</f>
-        <v/>
-      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5423,19 +4816,6 @@
       <c r="C49" t="inlineStr"/>
       <c r="D49">
         <f>SUMIF(J3:J47,"",D3:D47)</f>
-        <v/>
-      </c>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49">
-        <f>SUMIF(M3:M47,"",D3:D47)</f>
         <v/>
       </c>
     </row>
@@ -5450,7 +4830,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N40"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5463,10 +4843,8 @@
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5537,16 +4915,6 @@
           <t>Cost - new pigs (USD)</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
-        <is>
-          <t>Rate - unrated pigs at Pin (USD)</t>
-        </is>
-      </c>
-      <c r="N2" s="3" t="inlineStr">
-        <is>
-          <t>Cost - new pigs, unrated at Pin rate (USD)</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5585,20 +4953,13 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>pigs.xlsx Pin rate, same size</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L3" s="4">
         <f>IF(J3="","",D3*J3)</f>
         <v/>
       </c>
-      <c r="M3" s="4" t="n">
-        <v>53.1</v>
-      </c>
-      <c r="N3" s="4">
-        <f>IF(M3="","",D3*M3)</f>
-        <v/>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
@@ -5644,13 +5005,6 @@
         <f>IF(J4="","",D4*J4)</f>
         <v/>
       </c>
-      <c r="M4" s="9" t="n">
-        <v>53.1</v>
-      </c>
-      <c r="N4" s="9">
-        <f>IF(M4="","",D4*M4)</f>
-        <v/>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5694,11 +5048,6 @@
         <f>IF(J5="","",D5*J5)</f>
         <v/>
       </c>
-      <c r="M5" s="4" t="n"/>
-      <c r="N5" s="4">
-        <f>IF(M5="","",D5*M5)</f>
-        <v/>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
@@ -5744,13 +5093,6 @@
         <f>IF(J6="","",D6*J6)</f>
         <v/>
       </c>
-      <c r="M6" s="9" t="n">
-        <v>53.1</v>
-      </c>
-      <c r="N6" s="9">
-        <f>IF(M6="","",D6*M6)</f>
-        <v/>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -5796,13 +5138,6 @@
         <f>IF(J7="","",D7*J7)</f>
         <v/>
       </c>
-      <c r="M7" s="4" t="n">
-        <v>18.9</v>
-      </c>
-      <c r="N7" s="4">
-        <f>IF(M7="","",D7*M7)</f>
-        <v/>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
@@ -5848,13 +5183,6 @@
         <f>IF(J8="","",D8*J8)</f>
         <v/>
       </c>
-      <c r="M8" s="9" t="n">
-        <v>18.9</v>
-      </c>
-      <c r="N8" s="9">
-        <f>IF(M8="","",D8*M8)</f>
-        <v/>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5893,20 +5221,13 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>pigs.xlsx Pin rate, same size</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L9" s="4">
         <f>IF(J9="","",D9*J9)</f>
         <v/>
       </c>
-      <c r="M9" s="4" t="n">
-        <v>59</v>
-      </c>
-      <c r="N9" s="4">
-        <f>IF(M9="","",D9*M9)</f>
-        <v/>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
@@ -5952,13 +5273,6 @@
         <f>IF(J10="","",D10*J10)</f>
         <v/>
       </c>
-      <c r="M10" s="9" t="n">
-        <v>59</v>
-      </c>
-      <c r="N10" s="9">
-        <f>IF(M10="","",D10*M10)</f>
-        <v/>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -6002,11 +5316,6 @@
         <f>IF(J11="","",D11*J11)</f>
         <v/>
       </c>
-      <c r="M11" s="4" t="n"/>
-      <c r="N11" s="4">
-        <f>IF(M11="","",D11*M11)</f>
-        <v/>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
@@ -6052,13 +5361,6 @@
         <f>IF(J12="","",D12*J12)</f>
         <v/>
       </c>
-      <c r="M12" s="9" t="n">
-        <v>59</v>
-      </c>
-      <c r="N12" s="9">
-        <f>IF(M12="","",D12*M12)</f>
-        <v/>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6104,13 +5406,6 @@
         <f>IF(J13="","",D13*J13)</f>
         <v/>
       </c>
-      <c r="M13" s="4" t="n">
-        <v>59</v>
-      </c>
-      <c r="N13" s="4">
-        <f>IF(M13="","",D13*M13)</f>
-        <v/>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
@@ -6149,20 +5444,13 @@
       </c>
       <c r="K14" s="8" t="inlineStr">
         <is>
-          <t>pigs.xlsx Pin rate, same size</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L14" s="9">
         <f>IF(J14="","",D14*J14)</f>
         <v/>
       </c>
-      <c r="M14" s="9" t="n">
-        <v>64.90000000000001</v>
-      </c>
-      <c r="N14" s="9">
-        <f>IF(M14="","",D14*M14)</f>
-        <v/>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -6208,13 +5496,6 @@
         <f>IF(J15="","",D15*J15)</f>
         <v/>
       </c>
-      <c r="M15" s="4" t="n">
-        <v>64.90000000000001</v>
-      </c>
-      <c r="N15" s="4">
-        <f>IF(M15="","",D15*M15)</f>
-        <v/>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
@@ -6258,11 +5539,6 @@
         <f>IF(J16="","",D16*J16)</f>
         <v/>
       </c>
-      <c r="M16" s="9" t="n"/>
-      <c r="N16" s="9">
-        <f>IF(M16="","",D16*M16)</f>
-        <v/>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -6306,11 +5582,6 @@
         <f>IF(J17="","",D17*J17)</f>
         <v/>
       </c>
-      <c r="M17" s="4" t="n"/>
-      <c r="N17" s="4">
-        <f>IF(M17="","",D17*M17)</f>
-        <v/>
-      </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
@@ -6354,11 +5625,6 @@
         <f>IF(J18="","",D18*J18)</f>
         <v/>
       </c>
-      <c r="M18" s="9" t="n"/>
-      <c r="N18" s="9">
-        <f>IF(M18="","",D18*M18)</f>
-        <v/>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -6404,13 +5670,6 @@
         <f>IF(J19="","",D19*J19)</f>
         <v/>
       </c>
-      <c r="M19" s="4" t="n">
-        <v>49.6</v>
-      </c>
-      <c r="N19" s="4">
-        <f>IF(M19="","",D19*M19)</f>
-        <v/>
-      </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
@@ -6456,13 +5715,6 @@
         <f>IF(J20="","",D20*J20)</f>
         <v/>
       </c>
-      <c r="M20" s="9" t="n">
-        <v>49.6</v>
-      </c>
-      <c r="N20" s="9">
-        <f>IF(M20="","",D20*M20)</f>
-        <v/>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -6496,23 +5748,18 @@
       <c r="I21" t="n">
         <v>0</v>
       </c>
-      <c r="J21" s="4" t="n"/>
+      <c r="J21" s="4" t="n">
+        <v>118</v>
+      </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>no rate (type not on pigs.xlsx)</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L21" s="4">
         <f>IF(J21="","",D21*J21)</f>
         <v/>
       </c>
-      <c r="M21" s="4" t="n">
-        <v>118</v>
-      </c>
-      <c r="N21" s="4">
-        <f>IF(M21="","",D21*M21)</f>
-        <v/>
-      </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
@@ -6558,13 +5805,6 @@
         <f>IF(J22="","",D22*J22)</f>
         <v/>
       </c>
-      <c r="M22" s="9" t="n">
-        <v>118</v>
-      </c>
-      <c r="N22" s="9">
-        <f>IF(M22="","",D22*M22)</f>
-        <v/>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -6610,13 +5850,6 @@
         <f>IF(J23="","",D23*J23)</f>
         <v/>
       </c>
-      <c r="M23" s="4" t="n">
-        <v>129.8</v>
-      </c>
-      <c r="N23" s="4">
-        <f>IF(M23="","",D23*M23)</f>
-        <v/>
-      </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
@@ -6660,11 +5893,6 @@
         <f>IF(J24="","",D24*J24)</f>
         <v/>
       </c>
-      <c r="M24" s="9" t="n"/>
-      <c r="N24" s="9">
-        <f>IF(M24="","",D24*M24)</f>
-        <v/>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -6710,13 +5938,6 @@
         <f>IF(J25="","",D25*J25)</f>
         <v/>
       </c>
-      <c r="M25" s="4" t="n">
-        <v>129.8</v>
-      </c>
-      <c r="N25" s="4">
-        <f>IF(M25="","",D25*M25)</f>
-        <v/>
-      </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
@@ -6755,20 +5976,13 @@
       </c>
       <c r="K26" s="8" t="inlineStr">
         <is>
-          <t>pigs.xlsx Pin rate, same size</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L26" s="9">
         <f>IF(J26="","",D26*J26)</f>
         <v/>
       </c>
-      <c r="M26" s="9" t="n">
-        <v>230.1</v>
-      </c>
-      <c r="N26" s="9">
-        <f>IF(M26="","",D26*M26)</f>
-        <v/>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6812,11 +6026,6 @@
         <f>IF(J27="","",D27*J27)</f>
         <v/>
       </c>
-      <c r="M27" s="4" t="n"/>
-      <c r="N27" s="4">
-        <f>IF(M27="","",D27*M27)</f>
-        <v/>
-      </c>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
@@ -6862,13 +6071,6 @@
         <f>IF(J28="","",D28*J28)</f>
         <v/>
       </c>
-      <c r="M28" s="9" t="n">
-        <v>247.8</v>
-      </c>
-      <c r="N28" s="9">
-        <f>IF(M28="","",D28*M28)</f>
-        <v/>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -6914,13 +6116,6 @@
         <f>IF(J29="","",D29*J29)</f>
         <v/>
       </c>
-      <c r="M29" s="4" t="n">
-        <v>247.8</v>
-      </c>
-      <c r="N29" s="4">
-        <f>IF(M29="","",D29*M29)</f>
-        <v/>
-      </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
@@ -6959,20 +6154,13 @@
       </c>
       <c r="K30" s="8" t="inlineStr">
         <is>
-          <t>pigs.xlsx Pin rate, same size</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L30" s="9">
         <f>IF(J30="","",D30*J30)</f>
         <v/>
       </c>
-      <c r="M30" s="9" t="n">
-        <v>483.8</v>
-      </c>
-      <c r="N30" s="9">
-        <f>IF(M30="","",D30*M30)</f>
-        <v/>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -7018,13 +6206,6 @@
         <f>IF(J31="","",D31*J31)</f>
         <v/>
       </c>
-      <c r="M31" s="4" t="n">
-        <v>483.8</v>
-      </c>
-      <c r="N31" s="4">
-        <f>IF(M31="","",D31*M31)</f>
-        <v/>
-      </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
@@ -7070,13 +6251,6 @@
         <f>IF(J32="","",D32*J32)</f>
         <v/>
       </c>
-      <c r="M32" s="9" t="n">
-        <v>26.5</v>
-      </c>
-      <c r="N32" s="9">
-        <f>IF(M32="","",D32*M32)</f>
-        <v/>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -7120,11 +6294,6 @@
         <f>IF(J33="","",D33*J33)</f>
         <v/>
       </c>
-      <c r="M33" s="4" t="n"/>
-      <c r="N33" s="4">
-        <f>IF(M33="","",D33*M33)</f>
-        <v/>
-      </c>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
@@ -7163,20 +6332,13 @@
       </c>
       <c r="K34" s="8" t="inlineStr">
         <is>
-          <t>pigs.xlsx Pin rate, same size</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L34" s="9">
         <f>IF(J34="","",D34*J34)</f>
         <v/>
       </c>
-      <c r="M34" s="9" t="n">
-        <v>826</v>
-      </c>
-      <c r="N34" s="9">
-        <f>IF(M34="","",D34*M34)</f>
-        <v/>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -7222,13 +6384,6 @@
         <f>IF(J35="","",D35*J35)</f>
         <v/>
       </c>
-      <c r="M35" s="4" t="n">
-        <v>826</v>
-      </c>
-      <c r="N35" s="4">
-        <f>IF(M35="","",D35*M35)</f>
-        <v/>
-      </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
@@ -7272,11 +6427,6 @@
         <f>IF(J36="","",D36*J36)</f>
         <v/>
       </c>
-      <c r="M36" s="9" t="n"/>
-      <c r="N36" s="9">
-        <f>IF(M36="","",D36*M36)</f>
-        <v/>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -7320,11 +6470,6 @@
         <f>IF(J37="","",D37*J37)</f>
         <v/>
       </c>
-      <c r="M37" s="4" t="n"/>
-      <c r="N37" s="4">
-        <f>IF(M37="","",D37*M37)</f>
-        <v/>
-      </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
@@ -7366,11 +6511,6 @@
       </c>
       <c r="L38" s="9">
         <f>IF(J38="","",D38*J38)</f>
-        <v/>
-      </c>
-      <c r="M38" s="9" t="n"/>
-      <c r="N38" s="9">
-        <f>IF(M38="","",D38*M38)</f>
         <v/>
       </c>
     </row>
@@ -7415,11 +6555,6 @@
         <f>SUM(L3:L38)</f>
         <v/>
       </c>
-      <c r="M39" s="5" t="inlineStr"/>
-      <c r="N39" s="6">
-        <f>SUM(N3:N38)</f>
-        <v/>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -7431,19 +6566,6 @@
       <c r="C40" t="inlineStr"/>
       <c r="D40">
         <f>SUMIF(J3:J38,"",D3:D38)</f>
-        <v/>
-      </c>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40">
-        <f>SUMIF(M3:M38,"",D3:D38)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
[Lane 1] USA26046 pig counts: unlisted sizes round up to the next listed size (Jesse)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02-facilities/Cenovus/Lima-OH/USA26046-pig-counts.xlsx
+++ b/02-facilities/Cenovus/Lima-OH/USA26046-pig-counts.xlsx
@@ -733,7 +733,7 @@
     <row r="11" ht="60" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Costing: New pigs only; used pigs are not costed (Jesse, 2026-10-02). Rates are from pigs.xlsx for the same size and type. Any pig without its own rate is priced as Pin at the same size (Jesse, 2026-10-02: "Unrated are priced as PIN"). Foam takes the Gauge Foam rate; foams, swabs and honeycomb are not repriced as Pin. Sizes not on pigs.xlsx at all carry no rate and are counted in "New pigs with no rate".</t>
+          <t>Costing: New pigs only; used pigs are not costed (Jesse, 2026-10-02). Rates are from pigs.xlsx for the same size and type. Any pig without its own rate is priced as Pin (Jesse, 2026-10-02: "Unrated are priced as PIN"); foams use the Gauge Foam list and swabs the Swab list. A size not on the list rounds UP to the next listed size (Jesse, 2026-10-02). Only illegible sizes and sizes above the largest listed one stay unpriced.</t>
         </is>
       </c>
     </row>
@@ -870,10 +870,12 @@
       <c r="I3" t="n">
         <v>0</v>
       </c>
-      <c r="J3" s="4" t="n"/>
+      <c r="J3" s="4" t="n">
+        <v>118</v>
+      </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 6" Pin (priced as Pin)</t>
         </is>
       </c>
       <c r="L3" s="4">
@@ -913,10 +915,12 @@
       <c r="I4" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J4" s="9" t="n"/>
+      <c r="J4" s="9" t="n">
+        <v>118</v>
+      </c>
       <c r="K4" s="8" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 6" Pin (priced as Pin)</t>
         </is>
       </c>
       <c r="L4" s="9">
@@ -1406,10 +1410,12 @@
       <c r="I15" t="n">
         <v>0</v>
       </c>
-      <c r="J15" s="4" t="n"/>
+      <c r="J15" s="4" t="n">
+        <v>182.9</v>
+      </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 7.25" Pin (priced as Pin)</t>
         </is>
       </c>
       <c r="L15" s="4">
@@ -1449,10 +1455,12 @@
       <c r="I16" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J16" s="9" t="n"/>
+      <c r="J16" s="9" t="n">
+        <v>230.1</v>
+      </c>
       <c r="K16" s="8" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 8" Pin (priced as Pin)</t>
         </is>
       </c>
       <c r="L16" s="9">
@@ -1492,10 +1500,12 @@
       <c r="I17" t="n">
         <v>0</v>
       </c>
-      <c r="J17" s="4" t="n"/>
+      <c r="J17" s="4" t="n">
+        <v>230.1</v>
+      </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 8" Pin (priced as Pin)</t>
         </is>
       </c>
       <c r="L17" s="4">
@@ -1535,10 +1545,12 @@
       <c r="I18" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J18" s="9" t="n"/>
+      <c r="J18" s="9" t="n">
+        <v>230.1</v>
+      </c>
       <c r="K18" s="8" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 8" Pin</t>
         </is>
       </c>
       <c r="L18" s="9">
@@ -1851,7 +1863,7 @@
       <c r="J25" s="4" t="n"/>
       <c r="K25" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>no rate (above the largest listed gauge foam)</t>
         </is>
       </c>
       <c r="L25" s="4">
@@ -2029,7 +2041,7 @@
       <c r="J29" s="4" t="n"/>
       <c r="K29" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>no rate (above the largest listed swab)</t>
         </is>
       </c>
       <c r="L29" s="4">
@@ -2444,10 +2456,12 @@
       <c r="I7" t="n">
         <v>0</v>
       </c>
-      <c r="J7" s="4" t="n"/>
+      <c r="J7" s="4" t="n">
+        <v>82.59999999999999</v>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 8" Gauge Foam</t>
         </is>
       </c>
       <c r="L7" s="4">
@@ -2577,10 +2591,12 @@
       <c r="I10" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J10" s="9" t="n"/>
+      <c r="J10" s="9" t="n">
+        <v>182.9</v>
+      </c>
       <c r="K10" s="8" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 7.25" Pin (priced as Pin)</t>
         </is>
       </c>
       <c r="L10" s="9">
@@ -2815,10 +2831,12 @@
       <c r="I3" t="n">
         <v>0</v>
       </c>
-      <c r="J3" s="4" t="n"/>
+      <c r="J3" s="4" t="n">
+        <v>35.4</v>
+      </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 3.125" Pin (priced as Pin)</t>
         </is>
       </c>
       <c r="L3" s="4">
@@ -2858,10 +2876,12 @@
       <c r="I4" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J4" s="9" t="n"/>
+      <c r="J4" s="9" t="n">
+        <v>35.4</v>
+      </c>
       <c r="K4" s="8" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 3.125" Pin</t>
         </is>
       </c>
       <c r="L4" s="9">
@@ -2901,10 +2921,12 @@
       <c r="I5" t="n">
         <v>0</v>
       </c>
-      <c r="J5" s="4" t="n"/>
+      <c r="J5" s="4" t="n">
+        <v>35.4</v>
+      </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 3.125" Pin (priced as Pin)</t>
         </is>
       </c>
       <c r="L5" s="4">
@@ -2944,10 +2966,12 @@
       <c r="I6" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J6" s="9" t="n"/>
+      <c r="J6" s="9" t="n">
+        <v>35.4</v>
+      </c>
       <c r="K6" s="8" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 3.125" Pin</t>
         </is>
       </c>
       <c r="L6" s="9">
@@ -2987,10 +3011,12 @@
       <c r="I7" t="n">
         <v>0</v>
       </c>
-      <c r="J7" s="4" t="n"/>
+      <c r="J7" s="4" t="n">
+        <v>16.5</v>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 3.625" Gauge Foam</t>
         </is>
       </c>
       <c r="L7" s="4">
@@ -3300,10 +3326,12 @@
       <c r="I14" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J14" s="9" t="n"/>
+      <c r="J14" s="9" t="n">
+        <v>41.3</v>
+      </c>
       <c r="K14" s="8" t="inlineStr">
         <is>
-          <t>no rate (type not on pigs.xlsx)</t>
+          <t>rounded up to 3.325" Pin (priced as Pin)</t>
         </is>
       </c>
       <c r="L14" s="9">
@@ -3343,10 +3371,12 @@
       <c r="I15" t="n">
         <v>1</v>
       </c>
-      <c r="J15" s="4" t="n"/>
+      <c r="J15" s="4" t="n">
+        <v>47.2</v>
+      </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 3.5" Pin (priced as Pin)</t>
         </is>
       </c>
       <c r="L15" s="4">
@@ -3386,10 +3416,12 @@
       <c r="I16" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J16" s="9" t="n"/>
+      <c r="J16" s="9" t="n">
+        <v>47.2</v>
+      </c>
       <c r="K16" s="8" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 3.5" Pin (priced as Pin)</t>
         </is>
       </c>
       <c r="L16" s="9">
@@ -3609,10 +3641,12 @@
       <c r="I21" t="n">
         <v>3</v>
       </c>
-      <c r="J21" s="4" t="n"/>
+      <c r="J21" s="4" t="n">
+        <v>47.2</v>
+      </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 3.625" Pin (priced as Pin)</t>
         </is>
       </c>
       <c r="L21" s="4">
@@ -3652,10 +3686,12 @@
       <c r="I22" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J22" s="9" t="n"/>
+      <c r="J22" s="9" t="n">
+        <v>47.2</v>
+      </c>
       <c r="K22" s="8" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 3.625" Pin (priced as Pin)</t>
         </is>
       </c>
       <c r="L22" s="9">
@@ -3695,10 +3731,12 @@
       <c r="I23" t="n">
         <v>0</v>
       </c>
-      <c r="J23" s="4" t="n"/>
+      <c r="J23" s="4" t="n">
+        <v>47.2</v>
+      </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 3.625" Pin (priced as Pin)</t>
         </is>
       </c>
       <c r="L23" s="4">
@@ -3738,10 +3776,12 @@
       <c r="I24" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J24" s="9" t="n"/>
+      <c r="J24" s="9" t="n">
+        <v>47.2</v>
+      </c>
       <c r="K24" s="8" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 3.625" Pin</t>
         </is>
       </c>
       <c r="L24" s="9">
@@ -3961,10 +4001,12 @@
       <c r="I29" t="n">
         <v>0</v>
       </c>
-      <c r="J29" s="4" t="n"/>
+      <c r="J29" s="4" t="n">
+        <v>53.1</v>
+      </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 3.75" Pin</t>
         </is>
       </c>
       <c r="L29" s="4">
@@ -4049,10 +4091,12 @@
       <c r="I31" t="n">
         <v>0</v>
       </c>
-      <c r="J31" s="4" t="n"/>
+      <c r="J31" s="4" t="n">
+        <v>18.9</v>
+      </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 4" Gauge Foam</t>
         </is>
       </c>
       <c r="L31" s="4">
@@ -4092,10 +4136,12 @@
       <c r="I32" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J32" s="9" t="n"/>
+      <c r="J32" s="9" t="n">
+        <v>18.9</v>
+      </c>
       <c r="K32" s="8" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 4" Gauge Foam</t>
         </is>
       </c>
       <c r="L32" s="9">
@@ -4270,10 +4316,12 @@
       <c r="I36" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J36" s="9" t="n"/>
+      <c r="J36" s="9" t="n">
+        <v>18.9</v>
+      </c>
       <c r="K36" s="8" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 4" Gauge Foam</t>
         </is>
       </c>
       <c r="L36" s="9">
@@ -4313,10 +4361,12 @@
       <c r="I37" t="n">
         <v>0</v>
       </c>
-      <c r="J37" s="4" t="n"/>
+      <c r="J37" s="4" t="n">
+        <v>53.1</v>
+      </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 3.875" Pin (priced as Pin)</t>
         </is>
       </c>
       <c r="L37" s="4">
@@ -4356,10 +4406,12 @@
       <c r="I38" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J38" s="9" t="n"/>
+      <c r="J38" s="9" t="n">
+        <v>53.1</v>
+      </c>
       <c r="K38" s="8" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 3.875" Pin</t>
         </is>
       </c>
       <c r="L38" s="9">
@@ -4444,10 +4496,12 @@
       <c r="I40" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J40" s="9" t="n"/>
+      <c r="J40" s="9" t="n">
+        <v>18.9</v>
+      </c>
       <c r="K40" s="8" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 4" Gauge Foam</t>
         </is>
       </c>
       <c r="L40" s="9">
@@ -4532,10 +4586,12 @@
       <c r="I42" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J42" s="9" t="n"/>
+      <c r="J42" s="9" t="n">
+        <v>59</v>
+      </c>
       <c r="K42" s="8" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 4" Pin</t>
         </is>
       </c>
       <c r="L42" s="9">
@@ -4710,10 +4766,12 @@
       <c r="I46" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J46" s="9" t="n"/>
+      <c r="J46" s="9" t="n">
+        <v>16.1</v>
+      </c>
       <c r="K46" s="8" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 8.5" Swab</t>
         </is>
       </c>
       <c r="L46" s="9">
@@ -5038,10 +5096,12 @@
       <c r="I5" t="n">
         <v>0</v>
       </c>
-      <c r="J5" s="4" t="n"/>
+      <c r="J5" s="4" t="n">
+        <v>53.1</v>
+      </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 3.875" Pin</t>
         </is>
       </c>
       <c r="L5" s="4">
@@ -5306,10 +5366,12 @@
       <c r="I11" t="n">
         <v>0</v>
       </c>
-      <c r="J11" s="4" t="n"/>
+      <c r="J11" s="4" t="n">
+        <v>59</v>
+      </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 4.125" Pin (priced as Pin)</t>
         </is>
       </c>
       <c r="L11" s="4">
@@ -5529,10 +5591,12 @@
       <c r="I16" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J16" s="9" t="n"/>
+      <c r="J16" s="9" t="n">
+        <v>118</v>
+      </c>
       <c r="K16" s="8" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 6" Pin (priced as Pin)</t>
         </is>
       </c>
       <c r="L16" s="9">
@@ -5572,10 +5636,12 @@
       <c r="I17" t="n">
         <v>0</v>
       </c>
-      <c r="J17" s="4" t="n"/>
+      <c r="J17" s="4" t="n">
+        <v>118</v>
+      </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 6" Pin</t>
         </is>
       </c>
       <c r="L17" s="4">
@@ -5615,10 +5681,12 @@
       <c r="I18" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J18" s="9" t="n"/>
+      <c r="J18" s="9" t="n">
+        <v>118</v>
+      </c>
       <c r="K18" s="8" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 6" Pin</t>
         </is>
       </c>
       <c r="L18" s="9">
@@ -5883,10 +5951,12 @@
       <c r="I24" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J24" s="9" t="n"/>
+      <c r="J24" s="9" t="n">
+        <v>82.59999999999999</v>
+      </c>
       <c r="K24" s="8" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 8" Gauge Foam</t>
         </is>
       </c>
       <c r="L24" s="9">
@@ -6016,10 +6086,12 @@
       <c r="I27" t="n">
         <v>0</v>
       </c>
-      <c r="J27" s="4" t="n"/>
+      <c r="J27" s="4" t="n">
+        <v>16.1</v>
+      </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 8.5" Swab</t>
         </is>
       </c>
       <c r="L27" s="4">
@@ -6284,10 +6356,12 @@
       <c r="I33" t="n">
         <v>0</v>
       </c>
-      <c r="J33" s="4" t="n"/>
+      <c r="J33" s="4" t="n">
+        <v>826</v>
+      </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>rounded up to 12" Pin</t>
         </is>
       </c>
       <c r="L33" s="4">
@@ -6420,7 +6494,7 @@
       <c r="J36" s="9" t="n"/>
       <c r="K36" s="8" t="inlineStr">
         <is>
-          <t>no rate (size not on pigs.xlsx)</t>
+          <t>no rate (above the largest listed pin)</t>
         </is>
       </c>
       <c r="L36" s="9">

</xml_diff>

<commit_message>
[Lane 1] USA26046 pig counts: oversize pigs charged as 8in foam / 10in swab / 12in pin (Jesse)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02-facilities/Cenovus/Lima-OH/USA26046-pig-counts.xlsx
+++ b/02-facilities/Cenovus/Lima-OH/USA26046-pig-counts.xlsx
@@ -1860,10 +1860,12 @@
       <c r="I25" t="n">
         <v>0</v>
       </c>
-      <c r="J25" s="4" t="n"/>
+      <c r="J25" s="4" t="n">
+        <v>82.59999999999999</v>
+      </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>no rate (above the largest listed gauge foam)</t>
+          <t>above the list - charged as 8" Gauge Foam</t>
         </is>
       </c>
       <c r="L25" s="4">
@@ -2038,10 +2040,12 @@
       <c r="I29" t="n">
         <v>0</v>
       </c>
-      <c r="J29" s="4" t="n"/>
+      <c r="J29" s="4" t="n">
+        <v>26.5</v>
+      </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>no rate (above the largest listed swab)</t>
+          <t>above the list - charged as 10" Swab</t>
         </is>
       </c>
       <c r="L29" s="4">
@@ -6491,10 +6495,12 @@
       <c r="I36" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="J36" s="9" t="n"/>
+      <c r="J36" s="9" t="n">
+        <v>826</v>
+      </c>
       <c r="K36" s="8" t="inlineStr">
         <is>
-          <t>no rate (above the largest listed pin)</t>
+          <t>above the list - charged as 12" Pin</t>
         </is>
       </c>
       <c r="L36" s="9">

</xml_diff>

<commit_message>
[Lane 1] USA26046 pig counts: six unsized pigs sized by Jesse; every new pig now priced
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02-facilities/Cenovus/Lima-OH/USA26046-pig-counts.xlsx
+++ b/02-facilities/Cenovus/Lima-OH/USA26046-pig-counts.xlsx
@@ -571,11 +571,11 @@
         <v>25</v>
       </c>
       <c r="I5" s="4">
-        <f>'Crude'!L31</f>
+        <f>'Crude'!L30</f>
         <v/>
       </c>
       <c r="J5">
-        <f>'Crude'!D32</f>
+        <f>'Crude'!D31</f>
         <v/>
       </c>
     </row>
@@ -643,11 +643,11 @@
         <v>25</v>
       </c>
       <c r="I7" s="4">
-        <f>'Coker'!L48</f>
+        <f>'Coker'!L47</f>
         <v/>
       </c>
       <c r="J7">
-        <f>'Coker'!D49</f>
+        <f>'Coker'!D48</f>
         <v/>
       </c>
     </row>
@@ -679,11 +679,11 @@
         <v>5</v>
       </c>
       <c r="I8" s="4">
-        <f>'Vac'!L39</f>
+        <f>'Vac'!L38</f>
         <v/>
       </c>
       <c r="J8">
-        <f>'Vac'!D40</f>
+        <f>'Vac'!D39</f>
         <v/>
       </c>
     </row>
@@ -752,7 +752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -985,10 +985,10 @@
         </is>
       </c>
       <c r="C6" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" s="8" t="n">
         <v>4</v>
-      </c>
-      <c r="D6" s="8" t="n">
-        <v>3</v>
       </c>
       <c r="E6" s="8" t="n">
         <v>1</v>
@@ -997,7 +997,7 @@
         <v>0</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H6" s="8" t="n">
         <v>1</v>
@@ -2054,100 +2054,57 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="inlineStr">
-        <is>
-          <t>size not legible</t>
-        </is>
-      </c>
-      <c r="B30" s="8" t="inlineStr">
-        <is>
-          <t>Foam</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F30" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H30" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I30" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J30" s="9" t="n"/>
-      <c r="K30" s="8" t="inlineStr">
-        <is>
-          <t>no rate (size not legible)</t>
-        </is>
-      </c>
-      <c r="L30" s="9">
-        <f>IF(J30="","",D30*J30)</f>
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr"/>
+      <c r="C30" s="5">
+        <f>SUM(C3:C29)</f>
         <v/>
       </c>
+      <c r="D30" s="5">
+        <f>SUM(D3:D29)</f>
+        <v/>
+      </c>
+      <c r="E30" s="5">
+        <f>SUM(E3:E29)</f>
+        <v/>
+      </c>
+      <c r="F30" s="5">
+        <f>SUM(F3:F29)</f>
+        <v/>
+      </c>
+      <c r="G30" s="5">
+        <f>SUM(G3:G29)</f>
+        <v/>
+      </c>
+      <c r="H30" s="5">
+        <f>SUM(H3:H29)</f>
+        <v/>
+      </c>
+      <c r="I30" s="5">
+        <f>SUM(I3:I29)</f>
+        <v/>
+      </c>
+      <c r="J30" s="5" t="inlineStr"/>
+      <c r="K30" s="5" t="inlineStr"/>
+      <c r="L30" s="6">
+        <f>SUM(L3:L29)</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr"/>
-      <c r="C31" s="5">
-        <f>SUM(C3:C30)</f>
-        <v/>
-      </c>
-      <c r="D31" s="5">
-        <f>SUM(D3:D30)</f>
-        <v/>
-      </c>
-      <c r="E31" s="5">
-        <f>SUM(E3:E30)</f>
-        <v/>
-      </c>
-      <c r="F31" s="5">
-        <f>SUM(F3:F30)</f>
-        <v/>
-      </c>
-      <c r="G31" s="5">
-        <f>SUM(G3:G30)</f>
-        <v/>
-      </c>
-      <c r="H31" s="5">
-        <f>SUM(H3:H30)</f>
-        <v/>
-      </c>
-      <c r="I31" s="5">
-        <f>SUM(I3:I30)</f>
-        <v/>
-      </c>
-      <c r="J31" s="5" t="inlineStr"/>
-      <c r="K31" s="5" t="inlineStr"/>
-      <c r="L31" s="6">
-        <f>SUM(L3:L30)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A31" t="inlineStr">
         <is>
           <t>New pigs with no rate</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32">
-        <f>SUMIF(J3:J30,"",D3:D30)</f>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31">
+        <f>SUMIF(J3:J29,"",D3:D29)</f>
         <v/>
       </c>
     </row>
@@ -2256,36 +2213,36 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Foam</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
         <v>0</v>
-      </c>
-      <c r="H3" t="n">
-        <v>1</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>118</v>
+        <v>49.6</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>priced as Pin, same size</t>
+          <t>pigs.xlsx (Gauge Foam rate)</t>
         </is>
       </c>
       <c r="L3" s="4">
@@ -2301,26 +2258,26 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Pin / TC / PPS</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="C4" s="8" t="n">
         <v>2</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E4" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="8" t="n">
-        <v>2</v>
-      </c>
       <c r="H4" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4" s="8" t="n">
         <v>0</v>
@@ -2330,7 +2287,7 @@
       </c>
       <c r="K4" s="8" t="inlineStr">
         <is>
-          <t>pigs.xlsx</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L4" s="9">
@@ -2341,37 +2298,37 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>6.25"</t>
+          <t>6"</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Bolted</t>
+          <t>Pin / TC / PPS</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" t="n">
         <v>0</v>
       </c>
-      <c r="H5" t="n">
-        <v>6</v>
-      </c>
       <c r="I5" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>129.8</v>
+        <v>118</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -2391,36 +2348,36 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>FMJ</t>
+          <t>Bolted</t>
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="8" t="n">
-        <v>2</v>
-      </c>
       <c r="H6" s="8" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I6" s="8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J6" s="9" t="n">
         <v>129.8</v>
       </c>
       <c r="K6" s="8" t="inlineStr">
         <is>
-          <t>priced as Pin, same size</t>
+          <t>pigs.xlsx</t>
         </is>
       </c>
       <c r="L6" s="9">
@@ -2436,14 +2393,14 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Foam</t>
+          <t>FMJ</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
@@ -2452,7 +2409,7 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -2461,11 +2418,11 @@
         <v>0</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>82.59999999999999</v>
+        <v>129.8</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>rounded up to 8" Gauge Foam</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L7" s="4">
@@ -2481,14 +2438,14 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Other / unclear</t>
+          <t>Foam</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E8" s="8" t="n">
         <v>0</v>
@@ -2497,7 +2454,7 @@
         <v>0</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H8" s="8" t="n">
         <v>0</v>
@@ -2506,11 +2463,11 @@
         <v>0</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>129.8</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="K8" s="8" t="inlineStr">
         <is>
-          <t>priced as Pin, same size</t>
+          <t>rounded up to 8" Gauge Foam</t>
         </is>
       </c>
       <c r="L8" s="9">
@@ -2526,26 +2483,26 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Pin / TC / PPS</t>
+          <t>Other / unclear</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -2555,7 +2512,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>pigs.xlsx</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L9" s="4">
@@ -2566,41 +2523,41 @@
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>6.5"</t>
+          <t>6.25"</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Other / unclear</t>
+          <t>Pin / TC / PPS</t>
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>0</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H10" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I10" s="8" t="n">
         <v>0</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>182.9</v>
+        <v>129.8</v>
       </c>
       <c r="K10" s="8" t="inlineStr">
         <is>
-          <t>rounded up to 7.25" Pin (priced as Pin)</t>
+          <t>pigs.xlsx</t>
         </is>
       </c>
       <c r="L10" s="9">
@@ -2611,19 +2568,19 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>size not legible</t>
+          <t>6.5"</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Foam</t>
+          <t>Other / unclear</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
@@ -2632,7 +2589,7 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -2640,10 +2597,12 @@
       <c r="I11" t="n">
         <v>0</v>
       </c>
-      <c r="J11" s="4" t="n"/>
+      <c r="J11" s="4" t="n">
+        <v>182.9</v>
+      </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>no rate (size not legible)</t>
+          <t>rounded up to 7.25" Pin (priced as Pin)</t>
         </is>
       </c>
       <c r="L11" s="4">
@@ -2717,7 +2676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4075,10 +4034,10 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D31" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E31" t="n">
         <v>0</v>
@@ -4087,7 +4046,7 @@
         <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H31" t="n">
         <v>0</v>
@@ -4784,100 +4743,57 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>size not legible</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Foam</t>
-        </is>
-      </c>
-      <c r="C47" t="n">
-        <v>1</v>
-      </c>
-      <c r="D47" t="n">
-        <v>1</v>
-      </c>
-      <c r="E47" t="n">
-        <v>0</v>
-      </c>
-      <c r="F47" t="n">
-        <v>0</v>
-      </c>
-      <c r="G47" t="n">
-        <v>1</v>
-      </c>
-      <c r="H47" t="n">
-        <v>0</v>
-      </c>
-      <c r="I47" t="n">
-        <v>0</v>
-      </c>
-      <c r="J47" s="4" t="n"/>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>no rate (size not legible)</t>
-        </is>
-      </c>
-      <c r="L47" s="4">
-        <f>IF(J47="","",D47*J47)</f>
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr"/>
+      <c r="C47" s="5">
+        <f>SUM(C3:C46)</f>
         <v/>
       </c>
+      <c r="D47" s="5">
+        <f>SUM(D3:D46)</f>
+        <v/>
+      </c>
+      <c r="E47" s="5">
+        <f>SUM(E3:E46)</f>
+        <v/>
+      </c>
+      <c r="F47" s="5">
+        <f>SUM(F3:F46)</f>
+        <v/>
+      </c>
+      <c r="G47" s="5">
+        <f>SUM(G3:G46)</f>
+        <v/>
+      </c>
+      <c r="H47" s="5">
+        <f>SUM(H3:H46)</f>
+        <v/>
+      </c>
+      <c r="I47" s="5">
+        <f>SUM(I3:I46)</f>
+        <v/>
+      </c>
+      <c r="J47" s="5" t="inlineStr"/>
+      <c r="K47" s="5" t="inlineStr"/>
+      <c r="L47" s="6">
+        <f>SUM(L3:L46)</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="5" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B48" s="5" t="inlineStr"/>
-      <c r="C48" s="5">
-        <f>SUM(C3:C47)</f>
-        <v/>
-      </c>
-      <c r="D48" s="5">
-        <f>SUM(D3:D47)</f>
-        <v/>
-      </c>
-      <c r="E48" s="5">
-        <f>SUM(E3:E47)</f>
-        <v/>
-      </c>
-      <c r="F48" s="5">
-        <f>SUM(F3:F47)</f>
-        <v/>
-      </c>
-      <c r="G48" s="5">
-        <f>SUM(G3:G47)</f>
-        <v/>
-      </c>
-      <c r="H48" s="5">
-        <f>SUM(H3:H47)</f>
-        <v/>
-      </c>
-      <c r="I48" s="5">
-        <f>SUM(I3:I47)</f>
-        <v/>
-      </c>
-      <c r="J48" s="5" t="inlineStr"/>
-      <c r="K48" s="5" t="inlineStr"/>
-      <c r="L48" s="6">
-        <f>SUM(L3:L47)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A48" t="inlineStr">
         <is>
           <t>New pigs with no rate</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr"/>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49">
-        <f>SUMIF(J3:J47,"",D3:D47)</f>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48">
+        <f>SUMIF(J3:J46,"",D3:D46)</f>
         <v/>
       </c>
     </row>
@@ -4892,7 +4808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5530,22 +5446,22 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D15" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E15" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F15" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G15" t="n">
         <v>3</v>
       </c>
       <c r="H15" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
@@ -6196,41 +6112,41 @@
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>10"</t>
+          <t>8.25"</t>
         </is>
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Swab</t>
         </is>
       </c>
       <c r="C30" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E30" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G30" s="8" t="n">
         <v>1</v>
       </c>
       <c r="H30" s="8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I30" s="8" t="n">
         <v>0</v>
       </c>
       <c r="J30" s="9" t="n">
-        <v>483.8</v>
+        <v>16.1</v>
       </c>
       <c r="K30" s="8" t="inlineStr">
         <is>
-          <t>priced as Pin, same size</t>
+          <t>rounded up to 8.5" Swab</t>
         </is>
       </c>
       <c r="L30" s="9">
@@ -6246,26 +6162,26 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Pin / TC / PPS</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="C31" t="n">
+        <v>6</v>
+      </c>
+      <c r="D31" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" t="n">
         <v>4</v>
       </c>
-      <c r="D31" t="n">
-        <v>1</v>
-      </c>
-      <c r="E31" t="n">
-        <v>3</v>
-      </c>
       <c r="F31" t="n">
         <v>1</v>
       </c>
       <c r="G31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I31" t="n">
         <v>0</v>
@@ -6275,7 +6191,7 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>pigs.xlsx</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L31" s="4">
@@ -6291,32 +6207,32 @@
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Swab</t>
+          <t>Pin / TC / PPS</t>
         </is>
       </c>
       <c r="C32" s="8" t="n">
         <v>4</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E32" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F32" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F32" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G32" s="8" t="n">
-        <v>4</v>
-      </c>
       <c r="H32" s="8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I32" s="8" t="n">
         <v>0</v>
       </c>
       <c r="J32" s="9" t="n">
-        <v>26.5</v>
+        <v>483.8</v>
       </c>
       <c r="K32" s="8" t="inlineStr">
         <is>
@@ -6331,41 +6247,41 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>10.25"</t>
+          <t>10"</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Pin / TC / PPS</t>
+          <t>Swab</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D33" t="n">
+        <v>4</v>
+      </c>
+      <c r="E33" t="n">
         <v>0</v>
-      </c>
-      <c r="E33" t="n">
-        <v>1</v>
       </c>
       <c r="F33" t="n">
         <v>0</v>
       </c>
       <c r="G33" t="n">
+        <v>4</v>
+      </c>
+      <c r="H33" t="n">
         <v>0</v>
-      </c>
-      <c r="H33" t="n">
-        <v>1</v>
       </c>
       <c r="I33" t="n">
         <v>0</v>
       </c>
       <c r="J33" s="4" t="n">
-        <v>826</v>
+        <v>26.5</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>rounded up to 12" Pin</t>
+          <t>pigs.xlsx</t>
         </is>
       </c>
       <c r="L33" s="4">
@@ -6376,31 +6292,31 @@
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>12"</t>
+          <t>10.25"</t>
         </is>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Pin / TC / PPS</t>
         </is>
       </c>
       <c r="C34" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D34" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E34" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G34" s="8" t="n">
         <v>0</v>
       </c>
       <c r="H34" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I34" s="8" t="n">
         <v>0</v>
@@ -6410,7 +6326,7 @@
       </c>
       <c r="K34" s="8" t="inlineStr">
         <is>
-          <t>priced as Pin, same size</t>
+          <t>rounded up to 12" Pin</t>
         </is>
       </c>
       <c r="L34" s="9">
@@ -6426,7 +6342,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Pin / TC / PPS</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -6455,7 +6371,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>pigs.xlsx</t>
+          <t>priced as Pin, same size</t>
         </is>
       </c>
       <c r="L35" s="4">
@@ -6466,7 +6382,7 @@
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>12.25"</t>
+          <t>12"</t>
         </is>
       </c>
       <c r="B36" s="8" t="inlineStr">
@@ -6475,13 +6391,13 @@
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D36" s="8" t="n">
         <v>1</v>
       </c>
       <c r="E36" s="8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F36" s="8" t="n">
         <v>1</v>
@@ -6490,7 +6406,7 @@
         <v>0</v>
       </c>
       <c r="H36" s="8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I36" s="8" t="n">
         <v>0</v>
@@ -6500,7 +6416,7 @@
       </c>
       <c r="K36" s="8" t="inlineStr">
         <is>
-          <t>above the list - charged as 12" Pin</t>
+          <t>pigs.xlsx</t>
         </is>
       </c>
       <c r="L36" s="9">
@@ -6511,7 +6427,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>size not legible</t>
+          <t>12.25"</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6520,13 +6436,13 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D37" t="n">
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F37" t="n">
         <v>1</v>
@@ -6535,15 +6451,17 @@
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I37" t="n">
         <v>0</v>
       </c>
-      <c r="J37" s="4" t="n"/>
+      <c r="J37" s="4" t="n">
+        <v>826</v>
+      </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>no rate (size not legible)</t>
+          <t>above the list - charged as 12" Pin</t>
         </is>
       </c>
       <c r="L37" s="4">
@@ -6552,100 +6470,57 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="8" t="inlineStr">
-        <is>
-          <t>size not legible</t>
-        </is>
-      </c>
-      <c r="B38" s="8" t="inlineStr">
-        <is>
-          <t>Swab</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E38" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F38" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G38" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H38" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I38" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J38" s="9" t="n"/>
-      <c r="K38" s="8" t="inlineStr">
-        <is>
-          <t>no rate (size not legible)</t>
-        </is>
-      </c>
-      <c r="L38" s="9">
-        <f>IF(J38="","",D38*J38)</f>
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr"/>
+      <c r="C38" s="5">
+        <f>SUM(C3:C37)</f>
         <v/>
       </c>
+      <c r="D38" s="5">
+        <f>SUM(D3:D37)</f>
+        <v/>
+      </c>
+      <c r="E38" s="5">
+        <f>SUM(E3:E37)</f>
+        <v/>
+      </c>
+      <c r="F38" s="5">
+        <f>SUM(F3:F37)</f>
+        <v/>
+      </c>
+      <c r="G38" s="5">
+        <f>SUM(G3:G37)</f>
+        <v/>
+      </c>
+      <c r="H38" s="5">
+        <f>SUM(H3:H37)</f>
+        <v/>
+      </c>
+      <c r="I38" s="5">
+        <f>SUM(I3:I37)</f>
+        <v/>
+      </c>
+      <c r="J38" s="5" t="inlineStr"/>
+      <c r="K38" s="5" t="inlineStr"/>
+      <c r="L38" s="6">
+        <f>SUM(L3:L37)</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B39" s="5" t="inlineStr"/>
-      <c r="C39" s="5">
-        <f>SUM(C3:C38)</f>
-        <v/>
-      </c>
-      <c r="D39" s="5">
-        <f>SUM(D3:D38)</f>
-        <v/>
-      </c>
-      <c r="E39" s="5">
-        <f>SUM(E3:E38)</f>
-        <v/>
-      </c>
-      <c r="F39" s="5">
-        <f>SUM(F3:F38)</f>
-        <v/>
-      </c>
-      <c r="G39" s="5">
-        <f>SUM(G3:G38)</f>
-        <v/>
-      </c>
-      <c r="H39" s="5">
-        <f>SUM(H3:H38)</f>
-        <v/>
-      </c>
-      <c r="I39" s="5">
-        <f>SUM(I3:I38)</f>
-        <v/>
-      </c>
-      <c r="J39" s="5" t="inlineStr"/>
-      <c r="K39" s="5" t="inlineStr"/>
-      <c r="L39" s="6">
-        <f>SUM(L3:L38)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A39" t="inlineStr">
         <is>
           <t>New pigs with no rate</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr"/>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40">
-        <f>SUMIF(J3:J38,"",D3:D38)</f>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39">
+        <f>SUMIF(J3:J37,"",D3:D37)</f>
         <v/>
       </c>
     </row>
@@ -9564,7 +9439,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>size not legible</t>
+          <t>3.75"</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -9592,7 +9467,7 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>no size written; Push Foam col marked</t>
+          <t>no size written; Push Foam col marked; size 3.75" per Jesse 2026-10-02</t>
         </is>
       </c>
     </row>
@@ -17387,7 +17262,7 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>size not legible</t>
+          <t>6"</t>
         </is>
       </c>
       <c r="F205" t="inlineStr">
@@ -17415,7 +17290,7 @@
       </c>
       <c r="K205" t="inlineStr">
         <is>
-          <t>no size written; side: RIGHT struck through on header</t>
+          <t>no size written; side: RIGHT struck through on header; size 6" per Jesse 2026-10-02</t>
         </is>
       </c>
     </row>
@@ -28038,7 +27913,7 @@
       </c>
       <c r="E408" t="inlineStr">
         <is>
-          <t>size not legible</t>
+          <t>6"</t>
         </is>
       </c>
       <c r="F408" t="inlineStr">
@@ -28066,7 +27941,7 @@
       </c>
       <c r="K408" t="inlineStr">
         <is>
-          <t>08:00; Push Foam ticked; size not written</t>
+          <t>08:00; Push Foam ticked; size not written; size 6" per Jesse 2026-10-02</t>
         </is>
       </c>
     </row>
@@ -31652,7 +31527,7 @@
       </c>
       <c r="E478" t="inlineStr">
         <is>
-          <t>size not legible</t>
+          <t>4.25"</t>
         </is>
       </c>
       <c r="F478" t="inlineStr">
@@ -31680,7 +31555,7 @@
       </c>
       <c r="K478" t="inlineStr">
         <is>
-          <t>size digit hidden by folded page corner; time 6:00</t>
+          <t>size digit hidden by folded page corner; time 6:00; size 4.25" per Jesse 2026-10-02</t>
         </is>
       </c>
     </row>
@@ -31705,7 +31580,7 @@
       </c>
       <c r="E479" t="inlineStr">
         <is>
-          <t>size not legible</t>
+          <t>4.25"</t>
         </is>
       </c>
       <c r="F479" t="inlineStr">
@@ -31733,7 +31608,7 @@
       </c>
       <c r="K479" t="inlineStr">
         <is>
-          <t>size hidden by folded page corner; time 730</t>
+          <t>size hidden by folded page corner; time 730; size 4.25" per Jesse 2026-10-02</t>
         </is>
       </c>
     </row>
@@ -36956,7 +36831,7 @@
       </c>
       <c r="E582" t="inlineStr">
         <is>
-          <t>size not legible</t>
+          <t>8.25"</t>
         </is>
       </c>
       <c r="F582" t="inlineStr">
@@ -36984,7 +36859,7 @@
       </c>
       <c r="K582" t="inlineStr">
         <is>
-          <t>no size written</t>
+          <t>no size written; size 8.25" per Jesse 2026-10-02</t>
         </is>
       </c>
     </row>

</xml_diff>